<commit_message>
Add Python M1 Python Basics activities and assignments
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +77,36 @@
         <fgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F8E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D7CCC8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFD8DC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -90,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -129,6 +159,42 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -496,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2987,6 +3053,3084 @@
       <c r="E92" s="7" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/calculator-using-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Final Project</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>website-creation-part-1</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/website-creation-part-1/website-creation-part-1.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Get Your Projects</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>website-creation-part-2</t>
+        </is>
+      </c>
+      <c r="E94" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/website-creation-part-2/website-creation-part-2.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>Lesson 33 – Let World Know You</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>website-creation-part-3</t>
+        </is>
+      </c>
+      <c r="E95" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/website-creation-part-3/website-creation-part-3.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Calculator Part 1</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>bank-app-part-1</t>
+        </is>
+      </c>
+      <c r="E96" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/bank-app-part-1/bank-app-part-1.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>Lesson 35 – Calculator Part 2</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>bank-app-part-2</t>
+        </is>
+      </c>
+      <c r="E97" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/bank-app-part-2/bank-app-part-2.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>Lesson 36 – Let's Calculate</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>bank-app-part-3</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/bank-app-part-3/bank-app-part-3.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C99" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Final Project</t>
+        </is>
+      </c>
+      <c r="D99" s="16" t="inlineStr">
+        <is>
+          <t>navigation-bar</t>
+        </is>
+      </c>
+      <c r="E99" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-31/navigation-bar.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B100" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C100" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Final Project</t>
+        </is>
+      </c>
+      <c r="D100" s="16" t="inlineStr">
+        <is>
+          <t>banner-image</t>
+        </is>
+      </c>
+      <c r="E100" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-31/banner-image.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Get Your Projects</t>
+        </is>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>about-section</t>
+        </is>
+      </c>
+      <c r="E101" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-32/about-section.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C102" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Get Your Projects</t>
+        </is>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>project-section</t>
+        </is>
+      </c>
+      <c r="E102" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-32/project-section.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 33 – Let World Know You</t>
+        </is>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>social-media</t>
+        </is>
+      </c>
+      <c r="E103" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-33/social-media.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B104" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 33 – Let World Know You</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>project-section</t>
+        </is>
+      </c>
+      <c r="E104" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-33/project-section.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B105" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Calculator Part 1</t>
+        </is>
+      </c>
+      <c r="D105" s="16" t="inlineStr">
+        <is>
+          <t>structure-of-calculator</t>
+        </is>
+      </c>
+      <c r="E105" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-34/structure-of-calculator.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B106" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C106" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Calculator Part 1</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="inlineStr">
+        <is>
+          <t>decorate-the-calculator</t>
+        </is>
+      </c>
+      <c r="E106" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-34/decorate-the-calculator.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B107" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C107" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 35 – Calculator Part 2</t>
+        </is>
+      </c>
+      <c r="D107" s="16" t="inlineStr">
+        <is>
+          <t>decorate-the-calculator</t>
+        </is>
+      </c>
+      <c r="E107" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-35/decorate-the-calculator.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="16" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B108" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C108" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 36 – Let's Calculate</t>
+        </is>
+      </c>
+      <c r="D108" s="16" t="inlineStr">
+        <is>
+          <t>functioning-of-the-calculator</t>
+        </is>
+      </c>
+      <c r="E108" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-36/functioning-of-the-calculator.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Operators &amp; Data Types</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="inlineStr">
+        <is>
+          <t>number-swapping</t>
+        </is>
+      </c>
+      <c r="E109" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/number-swapping/number-swapping.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="18" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>exam-eligibility</t>
+        </is>
+      </c>
+      <c r="E110" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/exam-eligibility/exam-eligibility.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="18" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C111" s="18" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Loops</t>
+        </is>
+      </c>
+      <c r="D111" s="18" t="inlineStr">
+        <is>
+          <t>armstrong-number</t>
+        </is>
+      </c>
+      <c r="E111" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/armstrong-number/armstrong-number.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B112" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 37 – Intro to Python</t>
+        </is>
+      </c>
+      <c r="D112" s="20" t="inlineStr">
+        <is>
+          <t>introduction-to-replit</t>
+        </is>
+      </c>
+      <c r="E112" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-37/introduction-to-replit.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B113" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C113" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 37 – Intro to Python</t>
+        </is>
+      </c>
+      <c r="D113" s="20" t="inlineStr">
+        <is>
+          <t>even-odd-flowchart</t>
+        </is>
+      </c>
+      <c r="E113" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-37/even-odd-flowchart.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B114" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C114" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 37 – Intro to Python</t>
+        </is>
+      </c>
+      <c r="D114" s="20" t="inlineStr">
+        <is>
+          <t>welcome-to-the-world-of-programming</t>
+        </is>
+      </c>
+      <c r="E114" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-37/welcome-to-the-world-of-programming.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="18" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B115" s="18" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C115" s="18" t="inlineStr">
+        <is>
+          <t>Lesson 37 – Intro to Python</t>
+        </is>
+      </c>
+      <c r="D115" s="18" t="inlineStr">
+        <is>
+          <t>flowchart</t>
+        </is>
+      </c>
+      <c r="E115" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/flowchart/flowchart.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B116" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C116" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Operators &amp; Data Types</t>
+        </is>
+      </c>
+      <c r="D116" s="20" t="inlineStr">
+        <is>
+          <t>data-types</t>
+        </is>
+      </c>
+      <c r="E116" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/data-types.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B117" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Operators &amp; Data Types</t>
+        </is>
+      </c>
+      <c r="D117" s="20" t="inlineStr">
+        <is>
+          <t>python-operators</t>
+        </is>
+      </c>
+      <c r="E117" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/python-operators.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B118" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C118" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Operators &amp; Data Types</t>
+        </is>
+      </c>
+      <c r="D118" s="20" t="inlineStr">
+        <is>
+          <t>string-operations</t>
+        </is>
+      </c>
+      <c r="E118" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/string-operations.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B119" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Operators &amp; Data Types</t>
+        </is>
+      </c>
+      <c r="D119" s="20" t="inlineStr">
+        <is>
+          <t>number-swap</t>
+        </is>
+      </c>
+      <c r="E119" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/number-swap.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B120" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D120" s="20" t="inlineStr">
+        <is>
+          <t>odd-even</t>
+        </is>
+      </c>
+      <c r="E120" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/odd-even.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B121" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C121" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D121" s="20" t="inlineStr">
+        <is>
+          <t>bmi-calculator</t>
+        </is>
+      </c>
+      <c r="E121" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/bmi-calculator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B122" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C122" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D122" s="20" t="inlineStr">
+        <is>
+          <t>double-check-number</t>
+        </is>
+      </c>
+      <c r="E122" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/double-check-number.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B123" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C123" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D123" s="20" t="inlineStr">
+        <is>
+          <t>date-time-operations</t>
+        </is>
+      </c>
+      <c r="E123" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/date-time-operations.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B124" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C124" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Loops</t>
+        </is>
+      </c>
+      <c r="D124" s="20" t="inlineStr">
+        <is>
+          <t>table-of-23</t>
+        </is>
+      </c>
+      <c r="E124" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/table-of-23.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B125" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C125" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Loops</t>
+        </is>
+      </c>
+      <c r="D125" s="20" t="inlineStr">
+        <is>
+          <t>star-pattern</t>
+        </is>
+      </c>
+      <c r="E125" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/star-pattern.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B126" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C126" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Loops</t>
+        </is>
+      </c>
+      <c r="D126" s="20" t="inlineStr">
+        <is>
+          <t>natural-numbers-sum</t>
+        </is>
+      </c>
+      <c r="E126" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/natural-numbers-sum.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B127" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C127" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Loops</t>
+        </is>
+      </c>
+      <c r="D127" s="20" t="inlineStr">
+        <is>
+          <t>prime-number</t>
+        </is>
+      </c>
+      <c r="E127" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/prime-number.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B128" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C128" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Functions</t>
+        </is>
+      </c>
+      <c r="D128" s="20" t="inlineStr">
+        <is>
+          <t>introduce-yourself</t>
+        </is>
+      </c>
+      <c r="E128" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-41/introduce-yourself.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B129" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C129" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Functions</t>
+        </is>
+      </c>
+      <c r="D129" s="20" t="inlineStr">
+        <is>
+          <t>factorial</t>
+        </is>
+      </c>
+      <c r="E129" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-41/factorial.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B130" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C130" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Functions</t>
+        </is>
+      </c>
+      <c r="D130" s="20" t="inlineStr">
+        <is>
+          <t>calculator</t>
+        </is>
+      </c>
+      <c r="E130" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-41/calculator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="18" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B131" s="18" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C131" s="18" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Functions</t>
+        </is>
+      </c>
+      <c r="D131" s="18" t="inlineStr">
+        <is>
+          <t>fibonacci-series</t>
+        </is>
+      </c>
+      <c r="E131" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/fibonacci-series/fibonacci-series.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B132" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C132" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 42 – Intro to Turtle</t>
+        </is>
+      </c>
+      <c r="D132" s="20" t="inlineStr">
+        <is>
+          <t>square-on-a-canvas</t>
+        </is>
+      </c>
+      <c r="E132" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-42/square-on-a-canvas.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B133" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C133" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 42 – Intro to Turtle</t>
+        </is>
+      </c>
+      <c r="D133" s="20" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="E133" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-42/star.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="20" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B134" s="20" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C134" s="20" t="inlineStr">
+        <is>
+          <t>Lesson 42 – Intro to Turtle</t>
+        </is>
+      </c>
+      <c r="D134" s="20" t="inlineStr">
+        <is>
+          <t>rainbow-spiral</t>
+        </is>
+      </c>
+      <c r="E134" s="21" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-42/rainbow-spiral.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="18" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B135" s="18" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C135" s="18" t="inlineStr">
+        <is>
+          <t>Lesson 42 – Intro to Turtle</t>
+        </is>
+      </c>
+      <c r="D135" s="18" t="inlineStr">
+        <is>
+          <t>fun-with-shapes</t>
+        </is>
+      </c>
+      <c r="E135" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/fun-with-shapes/fun-with-shapes.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="12" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B136" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C136" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Data Structures 1</t>
+        </is>
+      </c>
+      <c r="D136" s="12" t="inlineStr">
+        <is>
+          <t>number-guessing-game</t>
+        </is>
+      </c>
+      <c r="E136" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/number-guessing-game/number-guessing-game.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="12" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B137" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C137" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Data Structures 2</t>
+        </is>
+      </c>
+      <c r="D137" s="12" t="inlineStr">
+        <is>
+          <t>tuple-to-list</t>
+        </is>
+      </c>
+      <c r="E137" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/tuple-to-list/tuple-to-list.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="12" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B138" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C138" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 45 – OOP 1</t>
+        </is>
+      </c>
+      <c r="D138" s="12" t="inlineStr">
+        <is>
+          <t>robot-introduction</t>
+        </is>
+      </c>
+      <c r="E138" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/robot-introduction/robot-introduction.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="12" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B139" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C139" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 46 – OOP 2</t>
+        </is>
+      </c>
+      <c r="D139" s="12" t="inlineStr">
+        <is>
+          <t>expression-class</t>
+        </is>
+      </c>
+      <c r="E139" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/expression-class/expression-class.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="12" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C140" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 47 – Inheritance &amp; Abstraction</t>
+        </is>
+      </c>
+      <c r="D140" s="12" t="inlineStr">
+        <is>
+          <t>polygon-area-calculator</t>
+        </is>
+      </c>
+      <c r="E140" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/polygon-area-calculator/polygon-area-calculator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="12" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B141" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C141" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 48 – Polymorphism &amp; Encaps.</t>
+        </is>
+      </c>
+      <c r="D141" s="12" t="inlineStr">
+        <is>
+          <t>pet-care-dashboard</t>
+        </is>
+      </c>
+      <c r="E141" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/pet-care-dashboard/pet-care-dashboard.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Data Structures 1</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>operations-on-list</t>
+        </is>
+      </c>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-43/operations-on-list.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Data Structures 1</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>operations-on-dictionary</t>
+        </is>
+      </c>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-43/operations-on-dictionary.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Data Structures 1</t>
+        </is>
+      </c>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>list-to-dictionary</t>
+        </is>
+      </c>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-43/list-to-dictionary.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Data Structures 2</t>
+        </is>
+      </c>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>operations-on-tuple</t>
+        </is>
+      </c>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/operations-on-tuple.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Data Structures 2</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>operations-on-set</t>
+        </is>
+      </c>
+      <c r="E146" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/operations-on-set.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B147" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Data Structures 2</t>
+        </is>
+      </c>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t>set-union</t>
+        </is>
+      </c>
+      <c r="E147" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/set-union.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B148" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C148" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Data Structures 2</t>
+        </is>
+      </c>
+      <c r="D148" s="6" t="inlineStr">
+        <is>
+          <t>set-intersection</t>
+        </is>
+      </c>
+      <c r="E148" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/set-intersection.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B149" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C149" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 45 – OOP 1</t>
+        </is>
+      </c>
+      <c r="D149" s="6" t="inlineStr">
+        <is>
+          <t>class-student</t>
+        </is>
+      </c>
+      <c r="E149" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/class-student.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 45 – OOP 1</t>
+        </is>
+      </c>
+      <c r="D150" s="6" t="inlineStr">
+        <is>
+          <t>class-student-ii</t>
+        </is>
+      </c>
+      <c r="E150" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/class-student-ii.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B151" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C151" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 45 – OOP 1</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>parrot-bird</t>
+        </is>
+      </c>
+      <c r="E151" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/parrot-bird.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B152" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C152" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 45 – OOP 1</t>
+        </is>
+      </c>
+      <c r="D152" s="6" t="inlineStr">
+        <is>
+          <t>parrot-bird-ii</t>
+        </is>
+      </c>
+      <c r="E152" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/parrot-bird-ii.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B153" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 46 – OOP 2</t>
+        </is>
+      </c>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>constructor-and-destructor</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-46/constructor-and-destructor.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B154" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 46 – OOP 2</t>
+        </is>
+      </c>
+      <c r="D154" s="6" t="inlineStr">
+        <is>
+          <t>library-management-system</t>
+        </is>
+      </c>
+      <c r="E154" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-46/library-management-system.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B155" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 47 – Inheritance &amp; Abstraction</t>
+        </is>
+      </c>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t>employee-details</t>
+        </is>
+      </c>
+      <c r="E155" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-47/employee-details.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B156" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 47 – Inheritance &amp; Abstraction</t>
+        </is>
+      </c>
+      <c r="D156" s="6" t="inlineStr">
+        <is>
+          <t>student-details</t>
+        </is>
+      </c>
+      <c r="E156" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-47/student-details.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B157" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C157" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 47 – Inheritance &amp; Abstraction</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>animal-class</t>
+        </is>
+      </c>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-47/animal-class.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B158" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 48 – Polymorphism &amp; Encaps.</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="inlineStr">
+        <is>
+          <t>polymorphism-implementation</t>
+        </is>
+      </c>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-48/polymorphism-implementation.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B159" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C159" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 48 – Polymorphism &amp; Encaps.</t>
+        </is>
+      </c>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t>encapsulation-implementation</t>
+        </is>
+      </c>
+      <c r="E159" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-48/encapsulation-implementation.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B160" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C160" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 49 – File Handling</t>
+        </is>
+      </c>
+      <c r="D160" s="12" t="inlineStr">
+        <is>
+          <t>file-handling-access-modes</t>
+        </is>
+      </c>
+      <c r="E160" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/file-handling-access-modes/file-handling-access-modes.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="12" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B161" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C161" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 50 – Operations on a File 1</t>
+        </is>
+      </c>
+      <c r="D161" s="12" t="inlineStr">
+        <is>
+          <t>file-handling-operations-part-1</t>
+        </is>
+      </c>
+      <c r="E161" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/file-handling-operations-part-1/file-handling-operations-part-1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="12" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B162" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C162" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 51 – Operations on a File 2</t>
+        </is>
+      </c>
+      <c r="D162" s="12" t="inlineStr">
+        <is>
+          <t>file-handling-operations-part-2</t>
+        </is>
+      </c>
+      <c r="E162" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/file-handling-operations-part-2/file-handling-operations-part-2.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="12" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B163" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C163" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 52 – Tkinter in Python</t>
+        </is>
+      </c>
+      <c r="D163" s="12" t="inlineStr">
+        <is>
+          <t>random-password-generator</t>
+        </is>
+      </c>
+      <c r="E163" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/random-password-generator/random-password-generator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="12" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B164" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C164" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 53 – Tkinter Widgets</t>
+        </is>
+      </c>
+      <c r="D164" s="12" t="inlineStr">
+        <is>
+          <t>rock-paper-scissor</t>
+        </is>
+      </c>
+      <c r="E164" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/rock-paper-scissor/rock-paper-scissor.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="12" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B165" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C165" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 54 – Denomination Calculator</t>
+        </is>
+      </c>
+      <c r="D165" s="12" t="inlineStr">
+        <is>
+          <t>rock-paper-scissor-gui</t>
+        </is>
+      </c>
+      <c r="E165" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/rock-paper-scissor-gui/rock-paper-scissor-gui.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B166" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C166" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 49 – File Handling</t>
+        </is>
+      </c>
+      <c r="D166" s="16" t="inlineStr">
+        <is>
+          <t>file-handling-operations-part-1</t>
+        </is>
+      </c>
+      <c r="E166" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/file-handling-operations-part-1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B167" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C167" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 49 – File Handling</t>
+        </is>
+      </c>
+      <c r="D167" s="16" t="inlineStr">
+        <is>
+          <t>file-handling-operations-part-2</t>
+        </is>
+      </c>
+      <c r="E167" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/file-handling-operations-part-2.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B168" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C168" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 49 – File Handling</t>
+        </is>
+      </c>
+      <c r="D168" s="16" t="inlineStr">
+        <is>
+          <t>lines-in-file</t>
+        </is>
+      </c>
+      <c r="E168" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/lines-in-file.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B169" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C169" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 49 – File Handling</t>
+        </is>
+      </c>
+      <c r="D169" s="16" t="inlineStr">
+        <is>
+          <t>append-content</t>
+        </is>
+      </c>
+      <c r="E169" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/append-content.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B170" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C170" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 50 – Operations on a File 1</t>
+        </is>
+      </c>
+      <c r="D170" s="16" t="inlineStr">
+        <is>
+          <t>read-operations-part-1</t>
+        </is>
+      </c>
+      <c r="E170" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/read-operations-part-1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B171" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C171" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 50 – Operations on a File 1</t>
+        </is>
+      </c>
+      <c r="D171" s="16" t="inlineStr">
+        <is>
+          <t>read-operations-part-2</t>
+        </is>
+      </c>
+      <c r="E171" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/read-operations-part-2.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B172" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C172" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 50 – Operations on a File 1</t>
+        </is>
+      </c>
+      <c r="D172" s="16" t="inlineStr">
+        <is>
+          <t>remove-lines</t>
+        </is>
+      </c>
+      <c r="E172" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/remove-lines.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B173" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C173" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 50 – Operations on a File 1</t>
+        </is>
+      </c>
+      <c r="D173" s="16" t="inlineStr">
+        <is>
+          <t>odd-lines</t>
+        </is>
+      </c>
+      <c r="E173" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/odd-lines.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B174" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C174" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 51 – Operations on a File 2</t>
+        </is>
+      </c>
+      <c r="D174" s="16" t="inlineStr">
+        <is>
+          <t>file-handling-operations-part-1</t>
+        </is>
+      </c>
+      <c r="E174" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/file-handling-operations-part-1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B175" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C175" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 51 – Operations on a File 2</t>
+        </is>
+      </c>
+      <c r="D175" s="16" t="inlineStr">
+        <is>
+          <t>file-handling-operations-part-2</t>
+        </is>
+      </c>
+      <c r="E175" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/file-handling-operations-part-2.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B176" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C176" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 51 – Operations on a File 2</t>
+        </is>
+      </c>
+      <c r="D176" s="16" t="inlineStr">
+        <is>
+          <t>duplicate-lines</t>
+        </is>
+      </c>
+      <c r="E176" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/duplicate-lines.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B177" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C177" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 51 – Operations on a File 2</t>
+        </is>
+      </c>
+      <c r="D177" s="16" t="inlineStr">
+        <is>
+          <t>file-merge</t>
+        </is>
+      </c>
+      <c r="E177" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/file-merge.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B178" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C178" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 52 – Tkinter in Python</t>
+        </is>
+      </c>
+      <c r="D178" s="16" t="inlineStr">
+        <is>
+          <t>tkinter-1</t>
+        </is>
+      </c>
+      <c r="E178" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-52/tkinter-1.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B179" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C179" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 52 – Tkinter in Python</t>
+        </is>
+      </c>
+      <c r="D179" s="16" t="inlineStr">
+        <is>
+          <t>tkinter-2</t>
+        </is>
+      </c>
+      <c r="E179" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-52/tkinter-2.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B180" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C180" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 53 – Tkinter Widgets</t>
+        </is>
+      </c>
+      <c r="D180" s="16" t="inlineStr">
+        <is>
+          <t>image-makes-it-better</t>
+        </is>
+      </c>
+      <c r="E180" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-53/image-makes-it-better.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B181" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C181" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 53 – Tkinter Widgets</t>
+        </is>
+      </c>
+      <c r="D181" s="16" t="inlineStr">
+        <is>
+          <t>alert-virus-detected</t>
+        </is>
+      </c>
+      <c r="E181" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-53/alert-virus-detected.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B182" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C182" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 53 – Tkinter Widgets</t>
+        </is>
+      </c>
+      <c r="D182" s="16" t="inlineStr">
+        <is>
+          <t>lets-top-a-window</t>
+        </is>
+      </c>
+      <c r="E182" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-53/lets-top-a-window.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="16" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B183" s="16" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C183" s="16" t="inlineStr">
+        <is>
+          <t>Lesson 54 – Denomination Calculator</t>
+        </is>
+      </c>
+      <c r="D183" s="16" t="inlineStr">
+        <is>
+          <t>denomination-calculator-using-tkinter</t>
+        </is>
+      </c>
+      <c r="E183" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-54/denomination-calculator-using-tkinter.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B184" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C184" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 1 – Intro to Python</t>
+        </is>
+      </c>
+      <c r="D184" s="22" t="inlineStr">
+        <is>
+          <t>my-first-python-profile</t>
+        </is>
+      </c>
+      <c r="E184" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/my-first-python-profile/my-first-python-profile.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B185" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C185" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 2 – Getting Started</t>
+        </is>
+      </c>
+      <c r="D185" s="22" t="inlineStr">
+        <is>
+          <t>my-coding-id-card</t>
+        </is>
+      </c>
+      <c r="E185" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/my-coding-id-card/my-coding-id-card.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B186" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C186" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 3 – Data Types</t>
+        </is>
+      </c>
+      <c r="D186" s="22" t="inlineStr">
+        <is>
+          <t>student-library-card</t>
+        </is>
+      </c>
+      <c r="E186" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/student-library-card/student-library-card.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B187" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C187" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 4 – Operators I</t>
+        </is>
+      </c>
+      <c r="D187" s="22" t="inlineStr">
+        <is>
+          <t>monthly-pocket-money-tracker</t>
+        </is>
+      </c>
+      <c r="E187" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/monthly-pocket-money-tracker/monthly-pocket-money-tracker.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B188" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C188" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D188" s="22" t="inlineStr">
+        <is>
+          <t>school-trip-eligibility-checker</t>
+        </is>
+      </c>
+      <c r="E188" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/school-trip-eligibility-checker/school-trip-eligibility-checker.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B189" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C189" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Operators II</t>
+        </is>
+      </c>
+      <c r="D189" s="22" t="inlineStr">
+        <is>
+          <t>weekend-plan-adviser</t>
+        </is>
+      </c>
+      <c r="E189" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/weekend-plan-adviser/weekend-plan-adviser.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B190" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C190" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Operators III</t>
+        </is>
+      </c>
+      <c r="D190" s="22" t="inlineStr">
+        <is>
+          <t>gadget-locker-check</t>
+        </is>
+      </c>
+      <c r="E190" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/gadget-locker-check/gadget-locker-check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="22" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B191" s="22" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C191" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python Challenge</t>
+        </is>
+      </c>
+      <c r="D191" s="22" t="inlineStr">
+        <is>
+          <t>exam-score-analyser</t>
+        </is>
+      </c>
+      <c r="E191" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/exam-score-analyser/exam-score-analyser.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B192" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C192" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 1 – Intro to Python</t>
+        </is>
+      </c>
+      <c r="D192" s="24" t="inlineStr">
+        <is>
+          <t>print-statements-and-comments</t>
+        </is>
+      </c>
+      <c r="E192" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/print-statements-and-comments.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B193" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C193" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 2 – Getting Started</t>
+        </is>
+      </c>
+      <c r="D193" s="24" t="inlineStr">
+        <is>
+          <t>welcome-to-the-world-of-coding</t>
+        </is>
+      </c>
+      <c r="E193" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/welcome-to-the-world-of-coding.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B194" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C194" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 2 – Getting Started</t>
+        </is>
+      </c>
+      <c r="D194" s="24" t="inlineStr">
+        <is>
+          <t>understanding-the-variables</t>
+        </is>
+      </c>
+      <c r="E194" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/understanding-the-variables.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B195" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C195" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 2 – Getting Started</t>
+        </is>
+      </c>
+      <c r="D195" s="24" t="inlineStr">
+        <is>
+          <t>keywords</t>
+        </is>
+      </c>
+      <c r="E195" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/keywords.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B196" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C196" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 3 – Data Types</t>
+        </is>
+      </c>
+      <c r="D196" s="24" t="inlineStr">
+        <is>
+          <t>secret-agent-name-badge</t>
+        </is>
+      </c>
+      <c r="E196" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/secret-agent-name-badge.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B197" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C197" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 4 – Operators I</t>
+        </is>
+      </c>
+      <c r="D197" s="24" t="inlineStr">
+        <is>
+          <t>farm-harvest-calculator</t>
+        </is>
+      </c>
+      <c r="E197" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/farm-harvest-calculator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B198" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C198" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D198" s="24" t="inlineStr">
+        <is>
+          <t>weather-outfit-picker</t>
+        </is>
+      </c>
+      <c r="E198" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/weather-outfit-picker.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B199" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C199" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Operators II</t>
+        </is>
+      </c>
+      <c r="D199" s="24" t="inlineStr">
+        <is>
+          <t>smart-school-day-planner</t>
+        </is>
+      </c>
+      <c r="E199" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/smart-school-day-planner.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B200" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C200" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Operators III</t>
+        </is>
+      </c>
+      <c r="D200" s="24" t="inlineStr">
+        <is>
+          <t>identity-operator</t>
+        </is>
+      </c>
+      <c r="E200" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/identity-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B201" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C201" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Operators III</t>
+        </is>
+      </c>
+      <c r="D201" s="24" t="inlineStr">
+        <is>
+          <t>bitwise-operator</t>
+        </is>
+      </c>
+      <c r="E201" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/bitwise-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B202" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C202" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Operators III</t>
+        </is>
+      </c>
+      <c r="D202" s="24" t="inlineStr">
+        <is>
+          <t>membership-operator</t>
+        </is>
+      </c>
+      <c r="E202" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/membership-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B203" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C203" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python Challenge</t>
+        </is>
+      </c>
+      <c r="D203" s="24" t="inlineStr">
+        <is>
+          <t>operator-precedence</t>
+        </is>
+      </c>
+      <c r="E203" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/operator-precedence.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B204" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C204" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python Challenge</t>
+        </is>
+      </c>
+      <c r="D204" s="24" t="inlineStr">
+        <is>
+          <t>divisible-number</t>
+        </is>
+      </c>
+      <c r="E204" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/divisible-number.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B205" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C205" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python Challenge</t>
+        </is>
+      </c>
+      <c r="D205" s="24" t="inlineStr">
+        <is>
+          <t>mean-value</t>
+        </is>
+      </c>
+      <c r="E205" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/mean-value.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B206" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C206" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python Challenge</t>
+        </is>
+      </c>
+      <c r="D206" s="24" t="inlineStr">
+        <is>
+          <t>average-speed</t>
+        </is>
+      </c>
+      <c r="E206" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/average-speed.py</t>
         </is>
       </c>
     </row>
@@ -3083,6 +6227,120 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E206" r:id="rId205"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Align Python M1 with the M1 activity and ACP submission list
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +107,11 @@
         <fgColor rgb="00CFD8DC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEDC8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -120,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -195,6 +200,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -562,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E206"/>
+  <dimension ref="A1:E222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5526,17 +5537,17 @@
       </c>
       <c r="C184" s="22" t="inlineStr">
         <is>
-          <t>Lesson 1 – Intro to Python</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D184" s="22" t="inlineStr">
         <is>
-          <t>my-first-python-profile</t>
+          <t>odd-even-flowchart</t>
         </is>
       </c>
       <c r="E184" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/my-first-python-profile/my-first-python-profile.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/odd-even-flowchart/odd-even-flowchart.py</t>
         </is>
       </c>
     </row>
@@ -5553,17 +5564,17 @@
       </c>
       <c r="C185" s="22" t="inlineStr">
         <is>
-          <t>Lesson 2 – Getting Started</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D185" s="22" t="inlineStr">
         <is>
-          <t>my-coding-id-card</t>
+          <t>storing-birthdays</t>
         </is>
       </c>
       <c r="E185" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/my-coding-id-card/my-coding-id-card.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/storing-birthdays/storing-birthdays.py</t>
         </is>
       </c>
     </row>
@@ -5580,17 +5591,17 @@
       </c>
       <c r="C186" s="22" t="inlineStr">
         <is>
-          <t>Lesson 3 – Data Types</t>
+          <t>Lesson 3 – Data types in python</t>
         </is>
       </c>
       <c r="D186" s="22" t="inlineStr">
         <is>
-          <t>student-library-card</t>
+          <t>congratulations-message</t>
         </is>
       </c>
       <c r="E186" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/student-library-card/student-library-card.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/congratulations-message/congratulations-message.py</t>
         </is>
       </c>
     </row>
@@ -5607,17 +5618,17 @@
       </c>
       <c r="C187" s="22" t="inlineStr">
         <is>
-          <t>Lesson 4 – Operators I</t>
+          <t>Lesson 4 – Python Operators – I</t>
         </is>
       </c>
       <c r="D187" s="22" t="inlineStr">
         <is>
-          <t>monthly-pocket-money-tracker</t>
+          <t>square-root</t>
         </is>
       </c>
       <c r="E187" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/monthly-pocket-money-tracker/monthly-pocket-money-tracker.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/square-root/square-root.py</t>
         </is>
       </c>
     </row>
@@ -5639,12 +5650,12 @@
       </c>
       <c r="D188" s="22" t="inlineStr">
         <is>
-          <t>school-trip-eligibility-checker</t>
+          <t>summer-times</t>
         </is>
       </c>
       <c r="E188" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/school-trip-eligibility-checker/school-trip-eligibility-checker.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/summer-times/summer-times.py</t>
         </is>
       </c>
     </row>
@@ -5661,17 +5672,17 @@
       </c>
       <c r="C189" s="22" t="inlineStr">
         <is>
-          <t>Lesson 6 – Operators II</t>
+          <t>Lesson 6 – Python Operator II</t>
         </is>
       </c>
       <c r="D189" s="22" t="inlineStr">
         <is>
-          <t>weekend-plan-adviser</t>
+          <t>checking-alphabets</t>
         </is>
       </c>
       <c r="E189" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/weekend-plan-adviser/weekend-plan-adviser.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/checking-alphabets/checking-alphabets.py</t>
         </is>
       </c>
     </row>
@@ -5688,17 +5699,17 @@
       </c>
       <c r="C190" s="22" t="inlineStr">
         <is>
-          <t>Lesson 7 – Operators III</t>
+          <t>Lesson 7 – Python Operators III</t>
         </is>
       </c>
       <c r="D190" s="22" t="inlineStr">
         <is>
-          <t>gadget-locker-check</t>
+          <t>ascii-value</t>
         </is>
       </c>
       <c r="E190" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/gadget-locker-check/gadget-locker-check.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/ascii-value/ascii-value.py</t>
         </is>
       </c>
     </row>
@@ -5715,17 +5726,17 @@
       </c>
       <c r="C191" s="22" t="inlineStr">
         <is>
-          <t>Lesson 8 – Python Challenge</t>
+          <t>Lesson 8 – Python challenge</t>
         </is>
       </c>
       <c r="D191" s="22" t="inlineStr">
         <is>
-          <t>exam-score-analyser</t>
+          <t>number-swap</t>
         </is>
       </c>
       <c r="E191" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/exam-score-analyser/exam-score-analyser.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/number-swap/number-swap.py</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5753,7 @@
       </c>
       <c r="C192" s="24" t="inlineStr">
         <is>
-          <t>Lesson 1 – Intro to Python</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D192" s="24" t="inlineStr">
@@ -5769,17 +5780,17 @@
       </c>
       <c r="C193" s="24" t="inlineStr">
         <is>
-          <t>Lesson 2 – Getting Started</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D193" s="24" t="inlineStr">
         <is>
-          <t>welcome-to-the-world-of-coding</t>
+          <t>algorithm</t>
         </is>
       </c>
       <c r="E193" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/welcome-to-the-world-of-coding.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/algorithm.py</t>
         </is>
       </c>
     </row>
@@ -5796,17 +5807,17 @@
       </c>
       <c r="C194" s="24" t="inlineStr">
         <is>
-          <t>Lesson 2 – Getting Started</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D194" s="24" t="inlineStr">
         <is>
-          <t>understanding-the-variables</t>
+          <t>flowchart</t>
         </is>
       </c>
       <c r="E194" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/understanding-the-variables.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/flowchart.py</t>
         </is>
       </c>
     </row>
@@ -5823,17 +5834,17 @@
       </c>
       <c r="C195" s="24" t="inlineStr">
         <is>
-          <t>Lesson 2 – Getting Started</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D195" s="24" t="inlineStr">
         <is>
-          <t>keywords</t>
+          <t>platform-introduction</t>
         </is>
       </c>
       <c r="E195" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/keywords.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/platform-introduction.py</t>
         </is>
       </c>
     </row>
@@ -5850,17 +5861,17 @@
       </c>
       <c r="C196" s="24" t="inlineStr">
         <is>
-          <t>Lesson 3 – Data Types</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D196" s="24" t="inlineStr">
         <is>
-          <t>secret-agent-name-badge</t>
+          <t>welcome-to-the-world-of-coding</t>
         </is>
       </c>
       <c r="E196" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/secret-agent-name-badge.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/welcome-to-the-world-of-coding.py</t>
         </is>
       </c>
     </row>
@@ -5877,17 +5888,17 @@
       </c>
       <c r="C197" s="24" t="inlineStr">
         <is>
-          <t>Lesson 4 – Operators I</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D197" s="24" t="inlineStr">
         <is>
-          <t>farm-harvest-calculator</t>
+          <t>understanding-the-variables</t>
         </is>
       </c>
       <c r="E197" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/farm-harvest-calculator.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/understanding-the-variables.py</t>
         </is>
       </c>
     </row>
@@ -5904,17 +5915,17 @@
       </c>
       <c r="C198" s="24" t="inlineStr">
         <is>
-          <t>Lesson 5 – Conditional Statements</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D198" s="24" t="inlineStr">
         <is>
-          <t>weather-outfit-picker</t>
+          <t>keywords</t>
         </is>
       </c>
       <c r="E198" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/weather-outfit-picker.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/keywords.py</t>
         </is>
       </c>
     </row>
@@ -5931,17 +5942,17 @@
       </c>
       <c r="C199" s="24" t="inlineStr">
         <is>
-          <t>Lesson 6 – Operators II</t>
+          <t>Lesson 3 – Data types in python</t>
         </is>
       </c>
       <c r="D199" s="24" t="inlineStr">
         <is>
-          <t>smart-school-day-planner</t>
+          <t>data-types</t>
         </is>
       </c>
       <c r="E199" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/smart-school-day-planner.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/data-types.py</t>
         </is>
       </c>
     </row>
@@ -5958,17 +5969,17 @@
       </c>
       <c r="C200" s="24" t="inlineStr">
         <is>
-          <t>Lesson 7 – Operators III</t>
+          <t>Lesson 3 – Data types in python</t>
         </is>
       </c>
       <c r="D200" s="24" t="inlineStr">
         <is>
-          <t>identity-operator</t>
+          <t>typecasting</t>
         </is>
       </c>
       <c r="E200" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/identity-operator.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/typecasting.py</t>
         </is>
       </c>
     </row>
@@ -5985,17 +5996,17 @@
       </c>
       <c r="C201" s="24" t="inlineStr">
         <is>
-          <t>Lesson 7 – Operators III</t>
+          <t>Lesson 3 – Data types in python</t>
         </is>
       </c>
       <c r="D201" s="24" t="inlineStr">
         <is>
-          <t>bitwise-operator</t>
+          <t>string-operation</t>
         </is>
       </c>
       <c r="E201" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/bitwise-operator.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/string-operation.py</t>
         </is>
       </c>
     </row>
@@ -6012,17 +6023,17 @@
       </c>
       <c r="C202" s="24" t="inlineStr">
         <is>
-          <t>Lesson 7 – Operators III</t>
+          <t>Lesson 4 – Python Operators – I</t>
         </is>
       </c>
       <c r="D202" s="24" t="inlineStr">
         <is>
-          <t>membership-operator</t>
+          <t>average</t>
         </is>
       </c>
       <c r="E202" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/membership-operator.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/average.py</t>
         </is>
       </c>
     </row>
@@ -6039,17 +6050,17 @@
       </c>
       <c r="C203" s="24" t="inlineStr">
         <is>
-          <t>Lesson 8 – Python Challenge</t>
+          <t>Lesson 4 – Python Operators – I</t>
         </is>
       </c>
       <c r="D203" s="24" t="inlineStr">
         <is>
-          <t>operator-precedence</t>
+          <t>count-the-notes</t>
         </is>
       </c>
       <c r="E203" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/operator-precedence.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/count-the-notes.py</t>
         </is>
       </c>
     </row>
@@ -6066,17 +6077,17 @@
       </c>
       <c r="C204" s="24" t="inlineStr">
         <is>
-          <t>Lesson 8 – Python Challenge</t>
+          <t>Lesson 4 – Python Operators – I</t>
         </is>
       </c>
       <c r="D204" s="24" t="inlineStr">
         <is>
-          <t>divisible-number</t>
+          <t>percentage-calculation</t>
         </is>
       </c>
       <c r="E204" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/divisible-number.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/percentage-calculation.py</t>
         </is>
       </c>
     </row>
@@ -6093,17 +6104,17 @@
       </c>
       <c r="C205" s="24" t="inlineStr">
         <is>
-          <t>Lesson 8 – Python Challenge</t>
+          <t>Lesson 5 – Conditional Statements</t>
         </is>
       </c>
       <c r="D205" s="24" t="inlineStr">
         <is>
-          <t>mean-value</t>
+          <t>conditional-statements</t>
         </is>
       </c>
       <c r="E205" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/mean-value.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/conditional-statements.py</t>
         </is>
       </c>
     </row>
@@ -6120,17 +6131,449 @@
       </c>
       <c r="C206" s="24" t="inlineStr">
         <is>
-          <t>Lesson 8 – Python Challenge</t>
+          <t>Lesson 5 – Conditional Statements</t>
         </is>
       </c>
       <c r="D206" s="24" t="inlineStr">
         <is>
+          <t>profit-loss</t>
+        </is>
+      </c>
+      <c r="E206" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/profit-loss.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B207" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C207" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D207" s="24" t="inlineStr">
+        <is>
+          <t>checking-the-number-greater-or-smaller</t>
+        </is>
+      </c>
+      <c r="E207" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/checking-the-number-greater-or-smaller.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B208" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C208" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D208" s="24" t="inlineStr">
+        <is>
+          <t>odd-even</t>
+        </is>
+      </c>
+      <c r="E208" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/odd-even.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B209" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C209" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D209" s="24" t="inlineStr">
+        <is>
+          <t>and-or-operator</t>
+        </is>
+      </c>
+      <c r="E209" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/and-or-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B210" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C210" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D210" s="24" t="inlineStr">
+        <is>
+          <t>not-equal-operator</t>
+        </is>
+      </c>
+      <c r="E210" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/not-equal-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B211" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C211" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D211" s="24" t="inlineStr">
+        <is>
+          <t>bmi-checker</t>
+        </is>
+      </c>
+      <c r="E211" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/bmi-checker.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B212" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C212" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Python Operators III</t>
+        </is>
+      </c>
+      <c r="D212" s="24" t="inlineStr">
+        <is>
+          <t>identity-operator</t>
+        </is>
+      </c>
+      <c r="E212" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/identity-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B213" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C213" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Python Operators III</t>
+        </is>
+      </c>
+      <c r="D213" s="24" t="inlineStr">
+        <is>
+          <t>bitwise-operator</t>
+        </is>
+      </c>
+      <c r="E213" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/bitwise-operator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B214" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C214" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Python Operators III</t>
+        </is>
+      </c>
+      <c r="D214" s="24" t="inlineStr">
+        <is>
+          <t>grading-system</t>
+        </is>
+      </c>
+      <c r="E214" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/grading-system.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B215" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C215" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python challenge</t>
+        </is>
+      </c>
+      <c r="D215" s="24" t="inlineStr">
+        <is>
+          <t>operator-precedence</t>
+        </is>
+      </c>
+      <c r="E215" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/operator-precedence.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B216" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C216" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python challenge</t>
+        </is>
+      </c>
+      <c r="D216" s="24" t="inlineStr">
+        <is>
+          <t>divisible-number</t>
+        </is>
+      </c>
+      <c r="E216" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/divisible-number.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B217" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C217" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python challenge</t>
+        </is>
+      </c>
+      <c r="D217" s="24" t="inlineStr">
+        <is>
+          <t>mean-value</t>
+        </is>
+      </c>
+      <c r="E217" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/mean-value.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B218" s="24" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C218" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python challenge</t>
+        </is>
+      </c>
+      <c r="D218" s="24" t="inlineStr">
+        <is>
           <t>average-speed</t>
         </is>
       </c>
-      <c r="E206" s="25" t="inlineStr">
+      <c r="E218" s="25" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/average-speed.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="26" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B219" s="26" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C219" s="26" t="inlineStr">
+        <is>
+          <t>Lesson 3 – Data types in python</t>
+        </is>
+      </c>
+      <c r="D219" s="26" t="inlineStr">
+        <is>
+          <t>secret-agent-name-badge</t>
+        </is>
+      </c>
+      <c r="E219" s="27" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-03/secret-agent-name-badge.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="26" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B220" s="26" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C220" s="26" t="inlineStr">
+        <is>
+          <t>Lesson 4 – Python Operators – I</t>
+        </is>
+      </c>
+      <c r="D220" s="26" t="inlineStr">
+        <is>
+          <t>farm-harvest-calculator</t>
+        </is>
+      </c>
+      <c r="E220" s="27" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-04/farm-harvest-calculator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="26" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B221" s="26" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C221" s="26" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D221" s="26" t="inlineStr">
+        <is>
+          <t>weather-outfit-picker</t>
+        </is>
+      </c>
+      <c r="E221" s="27" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-05/weather-outfit-picker.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="26" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B222" s="26" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C222" s="26" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D222" s="26" t="inlineStr">
+        <is>
+          <t>smart-school-day-planner</t>
+        </is>
+      </c>
+      <c r="E222" s="27" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-06/smart-school-day-planner.py</t>
         </is>
       </c>
     </row>
@@ -6341,6 +6784,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E204" r:id="rId203"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E205" r:id="rId204"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E222" r:id="rId221"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Key Python M1 tracker rows to the submission form questions in form order
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -99,12 +99,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D7CCC8"/>
+        <fgColor rgb="00CFD8DC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFD8DC"/>
+        <fgColor rgb="00D7CCC8"/>
       </patternFill>
     </fill>
     <fill>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E222"/>
+  <dimension ref="A1:F222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,6 +581,7 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -609,6 +610,11 @@
           <t>GitHub Link</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Form Question</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -636,6 +642,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m2/my-favourite-cartoon-character-page/my-favourite-cartoon-character-page.html</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -663,6 +670,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m2/my-weather-app-homepage/my-weather-app-homepage.html</t>
         </is>
       </c>
+      <c r="F3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -690,6 +698,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m2/my-restaurant-menu-card/my-restaurant-menu-card.html</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -717,6 +726,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m2/get-familiar-with-pseudo-classes/get-familiar-with-pseudo-classes.html</t>
         </is>
       </c>
+      <c r="F5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -744,6 +754,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m2/my-fitness-routine-cards/my-fitness-routine-cards.html</t>
         </is>
       </c>
+      <c r="F6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -771,6 +782,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m2/zoo-rescue-tracker/zoo-rescue-tracker.html</t>
         </is>
       </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -798,6 +810,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/assignments/unequal-grids/unequal-grids.html</t>
         </is>
       </c>
+      <c r="F8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -825,6 +838,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/assignments/decorate-your-content-using-bootstrap/decorate-your-content-using-bootstrap.html</t>
         </is>
       </c>
+      <c r="F9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -852,6 +866,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/assignments/create-a-hobby-section-with-container/create-a-hobby-section-with-container.html</t>
         </is>
       </c>
+      <c r="F10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -879,6 +894,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/assignments/create-a-slider/create-a-slider.html</t>
         </is>
       </c>
+      <c r="F11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -906,6 +922,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/assignments/create-different-pagination-using-bootstrap/create-different-pagination-using-bootstrap.html</t>
         </is>
       </c>
+      <c r="F12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -933,6 +950,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/assignments/create-a-portfolio/create-a-portfolio.html</t>
         </is>
       </c>
+      <c r="F13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -960,6 +978,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-13/my-first-grid.html</t>
         </is>
       </c>
+      <c r="F14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -987,6 +1006,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-13/lets-experiment-with-grid.html</t>
         </is>
       </c>
+      <c r="F15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1014,6 +1034,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-13/grids-for-desktop.html</t>
         </is>
       </c>
+      <c r="F16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1041,6 +1062,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-14/display-headings-small-dl.html</t>
         </is>
       </c>
+      <c r="F17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1068,6 +1090,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-14/mark-code.html</t>
         </is>
       </c>
+      <c r="F18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1095,6 +1118,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-14/bootstrap-typography.html</t>
         </is>
       </c>
+      <c r="F19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1122,6 +1146,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-15/containers.html</t>
         </is>
       </c>
+      <c r="F20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1149,6 +1174,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-15/container-fluid.html</t>
         </is>
       </c>
+      <c r="F21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1176,6 +1202,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-15/add-color-and-border.html</t>
         </is>
       </c>
+      <c r="F22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1203,6 +1230,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-16/jumbotron-and-buttons.html</t>
         </is>
       </c>
+      <c r="F23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1230,6 +1258,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-16/badges.html</t>
         </is>
       </c>
+      <c r="F24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1257,6 +1286,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-16/progress-bar.html</t>
         </is>
       </c>
+      <c r="F25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1284,6 +1314,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-17/cards.html</t>
         </is>
       </c>
+      <c r="F26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1311,6 +1342,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-17/spinner.html</t>
         </is>
       </c>
+      <c r="F27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1338,6 +1370,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-17/pagination.html</t>
         </is>
       </c>
+      <c r="F28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1365,6 +1398,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-18/carousel.html</t>
         </is>
       </c>
+      <c r="F29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1392,6 +1426,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-18/horizontal-scrollspy.html</t>
         </is>
       </c>
+      <c r="F30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1419,6 +1454,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m3/activities/lesson-18/create-a-portfolio-of-your-own.html</t>
         </is>
       </c>
+      <c r="F31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -1446,6 +1482,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/assignments/simple-calculator/simple-calculator.html</t>
         </is>
       </c>
+      <c r="F32" s="8" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -1473,6 +1510,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/assignments/multiplication-using-functions/multiplication-using-functions.html</t>
         </is>
       </c>
+      <c r="F33" s="8" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -1500,6 +1538,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/assignments/methods-and-loops/methods-and-loops.html</t>
         </is>
       </c>
+      <c r="F34" s="8" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -1527,6 +1566,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/assignments/sum-of-arguments/sum-of-arguments.html</t>
         </is>
       </c>
+      <c r="F35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -1554,6 +1594,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/assignments/object-data-structure-and-array/object-data-structure-and-array.html</t>
         </is>
       </c>
+      <c r="F36" s="8" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -1581,6 +1622,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/assignments/accessing-values-with-html-dom-structure/accessing-values-with-html-dom-structure.html</t>
         </is>
       </c>
+      <c r="F37" s="8" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -1608,6 +1650,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-19/syntax-guide-and-commenting.html</t>
         </is>
       </c>
+      <c r="F38" s="10" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -1635,6 +1678,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-19/variables.html</t>
         </is>
       </c>
+      <c r="F39" s="10" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -1662,6 +1706,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-19/statements.html</t>
         </is>
       </c>
+      <c r="F40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -1689,6 +1734,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-19/values-and-types.html</t>
         </is>
       </c>
+      <c r="F41" s="10" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -1716,6 +1762,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-19/use-of-operators.html</t>
         </is>
       </c>
+      <c r="F42" s="10" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -1743,6 +1790,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-20/functions-in-js.html</t>
         </is>
       </c>
+      <c r="F43" s="10" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
@@ -1770,6 +1818,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-20/parameters-and-optional-parameters.html</t>
         </is>
       </c>
+      <c r="F44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
@@ -1797,6 +1846,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-20/scope-of-variables-in-functions.html</t>
         </is>
       </c>
+      <c r="F45" s="10" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -1824,6 +1874,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-20/expression-function.html</t>
         </is>
       </c>
+      <c r="F46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -1851,6 +1902,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-21/methods-in-js.html</t>
         </is>
       </c>
+      <c r="F47" s="10" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -1878,6 +1930,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-21/test-methods-in-js.html</t>
         </is>
       </c>
+      <c r="F48" s="10" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -1905,6 +1958,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-21/loops-in-js.html</t>
         </is>
       </c>
+      <c r="F49" s="10" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -1932,6 +1986,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-21/switch-in-js.html</t>
         </is>
       </c>
+      <c r="F50" s="10" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -1959,6 +2014,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-22/objects-in-js.html</t>
         </is>
       </c>
+      <c r="F51" s="10" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -1986,6 +2042,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-22/properties-of-object.html</t>
         </is>
       </c>
+      <c r="F52" s="10" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -2013,6 +2070,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-22/built-in-math-objects-in-js.html</t>
         </is>
       </c>
+      <c r="F53" s="10" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -2040,6 +2098,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-22/arguments-object-in-js.html</t>
         </is>
       </c>
+      <c r="F54" s="10" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -2067,6 +2126,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-23/object-data-structure.html</t>
         </is>
       </c>
+      <c r="F55" s="10" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -2094,6 +2154,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-23/math-object.html</t>
         </is>
       </c>
+      <c r="F56" s="10" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -2121,6 +2182,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-23/array-in-js.html</t>
         </is>
       </c>
+      <c r="F57" s="10" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -2148,6 +2210,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-23/methods-in-array.html</t>
         </is>
       </c>
+      <c r="F58" s="10" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
@@ -2175,6 +2238,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-23/call-stack.html</t>
         </is>
       </c>
+      <c r="F59" s="10" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
@@ -2202,6 +2266,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-24/html-dom.html</t>
         </is>
       </c>
+      <c r="F60" s="10" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -2229,6 +2294,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-24/html-dom-structure.html</t>
         </is>
       </c>
+      <c r="F61" s="10" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -2256,6 +2322,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-24/js-as-external-file.html</t>
         </is>
       </c>
+      <c r="F62" s="10" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -2283,6 +2350,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-24/real-time-application-using-js.html</t>
         </is>
       </c>
+      <c r="F63" s="10" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -2310,6 +2378,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/print-random-numbers/print-random-numbers.html</t>
         </is>
       </c>
+      <c r="F64" s="12" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
@@ -2337,6 +2406,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/class-in-js/class-in-js.html</t>
         </is>
       </c>
+      <c r="F65" s="12" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
@@ -2364,6 +2434,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/map-and-arrange-an-array/map-and-arrange-an-array.html</t>
         </is>
       </c>
+      <c r="F66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
@@ -2391,6 +2462,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/handle-errors-in-js/handle-errors-in-js.html</t>
         </is>
       </c>
+      <c r="F67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
@@ -2418,6 +2490,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/asynchronous-functions-in-js/asynchronous-functions-in-js.html</t>
         </is>
       </c>
+      <c r="F68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -2445,6 +2518,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/data-types-in-detail.html</t>
         </is>
       </c>
+      <c r="F69" s="6" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
@@ -2472,6 +2546,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/let-and-const-keywords.html</t>
         </is>
       </c>
+      <c r="F70" s="6" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -2499,6 +2574,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/conditional-statements.html</t>
         </is>
       </c>
+      <c r="F71" s="6" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -2526,6 +2602,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/generate-random-numbers-using-a-while-loop.html</t>
         </is>
       </c>
+      <c r="F72" s="6" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -2553,6 +2630,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/purpose-of-this-keyword.html</t>
         </is>
       </c>
+      <c r="F73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -2580,6 +2658,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/js-class.html</t>
         </is>
       </c>
+      <c r="F74" s="6" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -2607,6 +2686,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/class-inheritance.html</t>
         </is>
       </c>
+      <c r="F75" s="6" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
@@ -2634,6 +2714,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/static-methods-in-class.html</t>
         </is>
       </c>
+      <c r="F76" s="6" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
@@ -2661,6 +2742,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/sort-and-reverse-strings.html</t>
         </is>
       </c>
+      <c r="F77" s="6" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -2688,6 +2770,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/sort-and-reverse-numbers.html</t>
         </is>
       </c>
+      <c r="F78" s="6" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
@@ -2715,6 +2798,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/map-an-array.html</t>
         </is>
       </c>
+      <c r="F79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
@@ -2742,6 +2826,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/evaluate-variables.html</t>
         </is>
       </c>
+      <c r="F80" s="6" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -2769,6 +2854,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/type-conversion.html</t>
         </is>
       </c>
+      <c r="F81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
@@ -2796,6 +2882,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/search-and-replace-string.html</t>
         </is>
       </c>
+      <c r="F82" s="6" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -2823,6 +2910,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/error-handling-in-js.html</t>
         </is>
       </c>
+      <c r="F83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
@@ -2850,6 +2938,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/arrow-function-in-js.html</t>
         </is>
       </c>
+      <c r="F84" s="6" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -2877,6 +2966,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/json-in-js.html</t>
         </is>
       </c>
+      <c r="F85" s="6" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
@@ -2904,6 +2994,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/callback-functions.html</t>
         </is>
       </c>
+      <c r="F86" s="6" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
@@ -2931,6 +3022,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/promises-in-js.html</t>
         </is>
       </c>
+      <c r="F87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
@@ -2958,6 +3050,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/async-await-in-js.html</t>
         </is>
       </c>
+      <c r="F88" s="6" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
@@ -2985,6 +3078,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/validate-inputs/validate-inputs.html</t>
         </is>
       </c>
+      <c r="F89" s="12" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
@@ -3012,6 +3106,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/form-validation.html</t>
         </is>
       </c>
+      <c r="F90" s="6" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
@@ -3039,6 +3134,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/validation-using-api.html</t>
         </is>
       </c>
+      <c r="F91" s="6" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
@@ -3066,6 +3162,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/calculator-using-js.html</t>
         </is>
       </c>
+      <c r="F92" s="6" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
@@ -3093,6 +3190,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/website-creation-part-1/website-creation-part-1.html</t>
         </is>
       </c>
+      <c r="F93" s="14" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
@@ -3120,6 +3218,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/website-creation-part-2/website-creation-part-2.html</t>
         </is>
       </c>
+      <c r="F94" s="14" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
@@ -3147,6 +3246,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/website-creation-part-3/website-creation-part-3.html</t>
         </is>
       </c>
+      <c r="F95" s="14" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
@@ -3174,6 +3274,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/bank-app-part-1/bank-app-part-1.html</t>
         </is>
       </c>
+      <c r="F96" s="14" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="14" t="inlineStr">
@@ -3201,6 +3302,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/bank-app-part-2/bank-app-part-2.html</t>
         </is>
       </c>
+      <c r="F97" s="14" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
@@ -3228,6 +3330,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/assignments/bank-app-part-3/bank-app-part-3.html</t>
         </is>
       </c>
+      <c r="F98" s="14" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -3255,6 +3358,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-31/navigation-bar.html</t>
         </is>
       </c>
+      <c r="F99" s="16" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -3282,6 +3386,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-31/banner-image.html</t>
         </is>
       </c>
+      <c r="F100" s="16" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
@@ -3309,6 +3414,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-32/about-section.html</t>
         </is>
       </c>
+      <c r="F101" s="16" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
@@ -3336,6 +3442,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-32/project-section.html</t>
         </is>
       </c>
+      <c r="F102" s="16" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
@@ -3363,6 +3470,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-33/social-media.html</t>
         </is>
       </c>
+      <c r="F103" s="16" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -3390,6 +3498,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-33/project-section.html</t>
         </is>
       </c>
+      <c r="F104" s="16" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -3417,6 +3526,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-34/structure-of-calculator.html</t>
         </is>
       </c>
+      <c r="F105" s="16" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -3444,6 +3554,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-34/decorate-the-calculator.html</t>
         </is>
       </c>
+      <c r="F106" s="16" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
@@ -3471,6 +3582,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-35/decorate-the-calculator.html</t>
         </is>
       </c>
+      <c r="F107" s="16" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
@@ -3498,6 +3610,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m6/activities/lesson-36/functioning-of-the-calculator.html</t>
         </is>
       </c>
+      <c r="F108" s="16" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="18" t="inlineStr">
@@ -3525,6 +3638,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/number-swapping/number-swapping.py</t>
         </is>
       </c>
+      <c r="F109" s="18" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="18" t="inlineStr">
@@ -3552,6 +3666,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/exam-eligibility/exam-eligibility.py</t>
         </is>
       </c>
+      <c r="F110" s="18" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="18" t="inlineStr">
@@ -3579,6 +3694,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/armstrong-number/armstrong-number.py</t>
         </is>
       </c>
+      <c r="F111" s="18" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="20" t="inlineStr">
@@ -3606,6 +3722,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-37/introduction-to-replit.py</t>
         </is>
       </c>
+      <c r="F112" s="20" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="20" t="inlineStr">
@@ -3633,6 +3750,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-37/even-odd-flowchart.py</t>
         </is>
       </c>
+      <c r="F113" s="20" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="20" t="inlineStr">
@@ -3660,6 +3778,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-37/welcome-to-the-world-of-programming.py</t>
         </is>
       </c>
+      <c r="F114" s="20" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="18" t="inlineStr">
@@ -3687,6 +3806,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/flowchart/flowchart.py</t>
         </is>
       </c>
+      <c r="F115" s="18" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="20" t="inlineStr">
@@ -3714,6 +3834,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/data-types.py</t>
         </is>
       </c>
+      <c r="F116" s="20" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="20" t="inlineStr">
@@ -3741,6 +3862,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/python-operators.py</t>
         </is>
       </c>
+      <c r="F117" s="20" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="20" t="inlineStr">
@@ -3768,6 +3890,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/string-operations.py</t>
         </is>
       </c>
+      <c r="F118" s="20" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="20" t="inlineStr">
@@ -3795,6 +3918,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-38/number-swap.py</t>
         </is>
       </c>
+      <c r="F119" s="20" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="20" t="inlineStr">
@@ -3822,6 +3946,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/odd-even.py</t>
         </is>
       </c>
+      <c r="F120" s="20" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="20" t="inlineStr">
@@ -3849,6 +3974,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/bmi-calculator.py</t>
         </is>
       </c>
+      <c r="F121" s="20" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="20" t="inlineStr">
@@ -3876,6 +4002,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/double-check-number.py</t>
         </is>
       </c>
+      <c r="F122" s="20" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="20" t="inlineStr">
@@ -3903,6 +4030,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-39/date-time-operations.py</t>
         </is>
       </c>
+      <c r="F123" s="20" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="20" t="inlineStr">
@@ -3930,6 +4058,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/table-of-23.py</t>
         </is>
       </c>
+      <c r="F124" s="20" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="20" t="inlineStr">
@@ -3957,6 +4086,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/star-pattern.py</t>
         </is>
       </c>
+      <c r="F125" s="20" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="20" t="inlineStr">
@@ -3984,6 +4114,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/natural-numbers-sum.py</t>
         </is>
       </c>
+      <c r="F126" s="20" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="20" t="inlineStr">
@@ -4011,6 +4142,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-40/prime-number.py</t>
         </is>
       </c>
+      <c r="F127" s="20" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="20" t="inlineStr">
@@ -4038,6 +4170,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-41/introduce-yourself.py</t>
         </is>
       </c>
+      <c r="F128" s="20" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="20" t="inlineStr">
@@ -4065,6 +4198,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-41/factorial.py</t>
         </is>
       </c>
+      <c r="F129" s="20" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="20" t="inlineStr">
@@ -4092,6 +4226,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-41/calculator.py</t>
         </is>
       </c>
+      <c r="F130" s="20" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="18" t="inlineStr">
@@ -4119,6 +4254,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/fibonacci-series/fibonacci-series.py</t>
         </is>
       </c>
+      <c r="F131" s="18" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="20" t="inlineStr">
@@ -4146,6 +4282,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-42/square-on-a-canvas.py</t>
         </is>
       </c>
+      <c r="F132" s="20" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="20" t="inlineStr">
@@ -4173,6 +4310,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-42/star.py</t>
         </is>
       </c>
+      <c r="F133" s="20" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="20" t="inlineStr">
@@ -4200,6 +4338,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/activities/lesson-42/rainbow-spiral.py</t>
         </is>
       </c>
+      <c r="F134" s="20" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="18" t="inlineStr">
@@ -4227,6 +4366,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m7/assignments/fun-with-shapes/fun-with-shapes.py</t>
         </is>
       </c>
+      <c r="F135" s="18" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
@@ -4254,6 +4394,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/number-guessing-game/number-guessing-game.py</t>
         </is>
       </c>
+      <c r="F136" s="12" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
@@ -4281,6 +4422,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/tuple-to-list/tuple-to-list.py</t>
         </is>
       </c>
+      <c r="F137" s="12" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
@@ -4308,6 +4450,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/robot-introduction/robot-introduction.py</t>
         </is>
       </c>
+      <c r="F138" s="12" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
@@ -4335,6 +4478,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/expression-class/expression-class.py</t>
         </is>
       </c>
+      <c r="F139" s="12" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
@@ -4362,6 +4506,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/polygon-area-calculator/polygon-area-calculator.py</t>
         </is>
       </c>
+      <c r="F140" s="12" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
@@ -4389,6 +4534,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/assignments/pet-care-dashboard/pet-care-dashboard.py</t>
         </is>
       </c>
+      <c r="F141" s="12" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
@@ -4416,6 +4562,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-43/operations-on-list.py</t>
         </is>
       </c>
+      <c r="F142" s="6" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
@@ -4443,6 +4590,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-43/operations-on-dictionary.py</t>
         </is>
       </c>
+      <c r="F143" s="6" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
@@ -4470,6 +4618,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-43/list-to-dictionary.py</t>
         </is>
       </c>
+      <c r="F144" s="6" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
@@ -4497,6 +4646,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/operations-on-tuple.py</t>
         </is>
       </c>
+      <c r="F145" s="6" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
@@ -4524,6 +4674,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/operations-on-set.py</t>
         </is>
       </c>
+      <c r="F146" s="6" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
@@ -4551,6 +4702,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/set-union.py</t>
         </is>
       </c>
+      <c r="F147" s="6" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
@@ -4578,6 +4730,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-44/set-intersection.py</t>
         </is>
       </c>
+      <c r="F148" s="6" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
@@ -4605,6 +4758,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/class-student.py</t>
         </is>
       </c>
+      <c r="F149" s="6" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
@@ -4632,6 +4786,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/class-student-ii.py</t>
         </is>
       </c>
+      <c r="F150" s="6" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
@@ -4659,6 +4814,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/parrot-bird.py</t>
         </is>
       </c>
+      <c r="F151" s="6" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
@@ -4686,6 +4842,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-45/parrot-bird-ii.py</t>
         </is>
       </c>
+      <c r="F152" s="6" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
@@ -4713,6 +4870,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-46/constructor-and-destructor.py</t>
         </is>
       </c>
+      <c r="F153" s="6" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
@@ -4740,6 +4898,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-46/library-management-system.py</t>
         </is>
       </c>
+      <c r="F154" s="6" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
@@ -4767,6 +4926,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-47/employee-details.py</t>
         </is>
       </c>
+      <c r="F155" s="6" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="6" t="inlineStr">
@@ -4794,6 +4954,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-47/student-details.py</t>
         </is>
       </c>
+      <c r="F156" s="6" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
@@ -4821,6 +4982,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-47/animal-class.py</t>
         </is>
       </c>
+      <c r="F157" s="6" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="6" t="inlineStr">
@@ -4848,6 +5010,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-48/polymorphism-implementation.py</t>
         </is>
       </c>
+      <c r="F158" s="6" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="6" t="inlineStr">
@@ -4875,6 +5038,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m8/activities/lesson-48/encapsulation-implementation.py</t>
         </is>
       </c>
+      <c r="F159" s="6" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="12" t="inlineStr">
@@ -4902,6 +5066,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/file-handling-access-modes/file-handling-access-modes.py</t>
         </is>
       </c>
+      <c r="F160" s="12" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="12" t="inlineStr">
@@ -4929,6 +5094,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/file-handling-operations-part-1/file-handling-operations-part-1.py</t>
         </is>
       </c>
+      <c r="F161" s="12" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="12" t="inlineStr">
@@ -4956,6 +5122,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/file-handling-operations-part-2/file-handling-operations-part-2.py</t>
         </is>
       </c>
+      <c r="F162" s="12" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="12" t="inlineStr">
@@ -4983,6 +5150,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/random-password-generator/random-password-generator.py</t>
         </is>
       </c>
+      <c r="F163" s="12" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="12" t="inlineStr">
@@ -5010,6 +5178,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/rock-paper-scissor/rock-paper-scissor.py</t>
         </is>
       </c>
+      <c r="F164" s="12" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="12" t="inlineStr">
@@ -5037,6 +5206,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/assignments/rock-paper-scissor-gui/rock-paper-scissor-gui.py</t>
         </is>
       </c>
+      <c r="F165" s="12" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="16" t="inlineStr">
@@ -5064,6 +5234,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/file-handling-operations-part-1.py</t>
         </is>
       </c>
+      <c r="F166" s="16" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="16" t="inlineStr">
@@ -5091,6 +5262,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/file-handling-operations-part-2.py</t>
         </is>
       </c>
+      <c r="F167" s="16" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="16" t="inlineStr">
@@ -5118,6 +5290,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/lines-in-file.py</t>
         </is>
       </c>
+      <c r="F168" s="16" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="16" t="inlineStr">
@@ -5145,6 +5318,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-49/append-content.py</t>
         </is>
       </c>
+      <c r="F169" s="16" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="16" t="inlineStr">
@@ -5172,6 +5346,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/read-operations-part-1.py</t>
         </is>
       </c>
+      <c r="F170" s="16" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="16" t="inlineStr">
@@ -5199,6 +5374,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/read-operations-part-2.py</t>
         </is>
       </c>
+      <c r="F171" s="16" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="16" t="inlineStr">
@@ -5226,6 +5402,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/remove-lines.py</t>
         </is>
       </c>
+      <c r="F172" s="16" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="16" t="inlineStr">
@@ -5253,6 +5430,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-50/odd-lines.py</t>
         </is>
       </c>
+      <c r="F173" s="16" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="16" t="inlineStr">
@@ -5280,6 +5458,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/file-handling-operations-part-1.py</t>
         </is>
       </c>
+      <c r="F174" s="16" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="16" t="inlineStr">
@@ -5307,6 +5486,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/file-handling-operations-part-2.py</t>
         </is>
       </c>
+      <c r="F175" s="16" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="16" t="inlineStr">
@@ -5334,6 +5514,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/duplicate-lines.py</t>
         </is>
       </c>
+      <c r="F176" s="16" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="16" t="inlineStr">
@@ -5361,6 +5542,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-51/file-merge.py</t>
         </is>
       </c>
+      <c r="F177" s="16" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="16" t="inlineStr">
@@ -5388,6 +5570,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-52/tkinter-1.py</t>
         </is>
       </c>
+      <c r="F178" s="16" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="16" t="inlineStr">
@@ -5415,6 +5598,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-52/tkinter-2.py</t>
         </is>
       </c>
+      <c r="F179" s="16" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="16" t="inlineStr">
@@ -5442,6 +5626,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-53/image-makes-it-better.py</t>
         </is>
       </c>
+      <c r="F180" s="16" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="16" t="inlineStr">
@@ -5469,6 +5654,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-53/alert-virus-detected.py</t>
         </is>
       </c>
+      <c r="F181" s="16" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="16" t="inlineStr">
@@ -5496,6 +5682,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-53/lets-top-a-window.py</t>
         </is>
       </c>
+      <c r="F182" s="16" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="16" t="inlineStr">
@@ -5523,6 +5710,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m9/activities/lesson-54/denomination-calculator-using-tkinter.py</t>
         </is>
       </c>
+      <c r="F183" s="16" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="22" t="inlineStr">
@@ -5532,7 +5720,7 @@
       </c>
       <c r="B184" s="22" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="C184" s="22" t="inlineStr">
@@ -5542,12 +5730,17 @@
       </c>
       <c r="D184" s="22" t="inlineStr">
         <is>
-          <t>odd-even-flowchart</t>
+          <t>print-statements-and-comments</t>
         </is>
       </c>
       <c r="E184" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/odd-even-flowchart/odd-even-flowchart.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/print-statements-and-comments.py</t>
+        </is>
+      </c>
+      <c r="F184" s="22" t="inlineStr">
+        <is>
+          <t>M1L1 Activity 1: Print Statements and Comments</t>
         </is>
       </c>
     </row>
@@ -5559,22 +5752,27 @@
       </c>
       <c r="B185" s="22" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="C185" s="22" t="inlineStr">
         <is>
-          <t>Lesson 2 – Getting started with programming</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D185" s="22" t="inlineStr">
         <is>
-          <t>storing-birthdays</t>
+          <t>algorithm</t>
         </is>
       </c>
       <c r="E185" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/storing-birthdays/storing-birthdays.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/algorithm.py</t>
+        </is>
+      </c>
+      <c r="F185" s="22" t="inlineStr">
+        <is>
+          <t>M1L1 Activity 2: Algorithm (Legacy Activity)</t>
         </is>
       </c>
     </row>
@@ -5586,22 +5784,27 @@
       </c>
       <c r="B186" s="22" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="C186" s="22" t="inlineStr">
         <is>
-          <t>Lesson 3 – Data types in python</t>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
         </is>
       </c>
       <c r="D186" s="22" t="inlineStr">
         <is>
-          <t>congratulations-message</t>
+          <t>flowchart</t>
         </is>
       </c>
       <c r="E186" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/congratulations-message/congratulations-message.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/flowchart.py</t>
+        </is>
+      </c>
+      <c r="F186" s="22" t="inlineStr">
+        <is>
+          <t>M1L1 Activity 3: Flowchart (Legacy Activity)</t>
         </is>
       </c>
     </row>
@@ -5613,49 +5816,59 @@
       </c>
       <c r="B187" s="22" t="inlineStr">
         <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C187" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
+        </is>
+      </c>
+      <c r="D187" s="22" t="inlineStr">
+        <is>
+          <t>platform-introduction</t>
+        </is>
+      </c>
+      <c r="E187" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/platform-introduction.py</t>
+        </is>
+      </c>
+      <c r="F187" s="22" t="inlineStr">
+        <is>
+          <t>M1L1 Activity 4: Platform introduction (Legacy Activity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="24" t="inlineStr">
+        <is>
+          <t>PY-M1</t>
+        </is>
+      </c>
+      <c r="B188" s="24" t="inlineStr">
+        <is>
           <t>ACP</t>
         </is>
       </c>
-      <c r="C187" s="22" t="inlineStr">
-        <is>
-          <t>Lesson 4 – Python Operators – I</t>
-        </is>
-      </c>
-      <c r="D187" s="22" t="inlineStr">
-        <is>
-          <t>square-root</t>
-        </is>
-      </c>
-      <c r="E187" s="23" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/square-root/square-root.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="22" t="inlineStr">
-        <is>
-          <t>PY-M1</t>
-        </is>
-      </c>
-      <c r="B188" s="22" t="inlineStr">
-        <is>
-          <t>ACP</t>
-        </is>
-      </c>
-      <c r="C188" s="22" t="inlineStr">
-        <is>
-          <t>Lesson 5 – Conditional Statements</t>
-        </is>
-      </c>
-      <c r="D188" s="22" t="inlineStr">
-        <is>
-          <t>summer-times</t>
-        </is>
-      </c>
-      <c r="E188" s="23" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/summer-times/summer-times.py</t>
+      <c r="C188" s="24" t="inlineStr">
+        <is>
+          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
+        </is>
+      </c>
+      <c r="D188" s="24" t="inlineStr">
+        <is>
+          <t>odd-even-flowchart</t>
+        </is>
+      </c>
+      <c r="E188" s="25" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/odd-even-flowchart/odd-even-flowchart.py</t>
+        </is>
+      </c>
+      <c r="F188" s="24" t="inlineStr">
+        <is>
+          <t>M1L1 ACP : odd even flowchart</t>
         </is>
       </c>
     </row>
@@ -5667,22 +5880,27 @@
       </c>
       <c r="B189" s="22" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="C189" s="22" t="inlineStr">
         <is>
-          <t>Lesson 6 – Python Operator II</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D189" s="22" t="inlineStr">
         <is>
-          <t>checking-alphabets</t>
+          <t>welcome-to-the-world-of-coding</t>
         </is>
       </c>
       <c r="E189" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/checking-alphabets/checking-alphabets.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/welcome-to-the-world-of-coding.py</t>
+        </is>
+      </c>
+      <c r="F189" s="22" t="inlineStr">
+        <is>
+          <t>M1L2 Activity 1: Welcome to the world of coding</t>
         </is>
       </c>
     </row>
@@ -5694,22 +5912,27 @@
       </c>
       <c r="B190" s="22" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="C190" s="22" t="inlineStr">
         <is>
-          <t>Lesson 7 – Python Operators III</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D190" s="22" t="inlineStr">
         <is>
-          <t>ascii-value</t>
+          <t>understanding-the-variables</t>
         </is>
       </c>
       <c r="E190" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/ascii-value/ascii-value.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/understanding-the-variables.py</t>
+        </is>
+      </c>
+      <c r="F190" s="22" t="inlineStr">
+        <is>
+          <t>M1L2 Activity 2: Understanding the variables</t>
         </is>
       </c>
     </row>
@@ -5721,22 +5944,27 @@
       </c>
       <c r="B191" s="22" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="C191" s="22" t="inlineStr">
         <is>
-          <t>Lesson 8 – Python challenge</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D191" s="22" t="inlineStr">
         <is>
-          <t>number-swap</t>
+          <t>keywords</t>
         </is>
       </c>
       <c r="E191" s="23" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/number-swap/number-swap.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/keywords.py</t>
+        </is>
+      </c>
+      <c r="F191" s="22" t="inlineStr">
+        <is>
+          <t>M1L2 Activity 3: Keywords</t>
         </is>
       </c>
     </row>
@@ -5748,103 +5976,123 @@
       </c>
       <c r="B192" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C192" s="24" t="inlineStr">
         <is>
-          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
+          <t>Lesson 2 – Getting started with programming</t>
         </is>
       </c>
       <c r="D192" s="24" t="inlineStr">
         <is>
-          <t>print-statements-and-comments</t>
+          <t>storing-birthdays</t>
         </is>
       </c>
       <c r="E192" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/print-statements-and-comments.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/storing-birthdays/storing-birthdays.py</t>
+        </is>
+      </c>
+      <c r="F192" s="24" t="inlineStr">
+        <is>
+          <t>M1L2 ACP : Storing birthdays</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="24" t="inlineStr">
+      <c r="A193" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B193" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C193" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
-        </is>
-      </c>
-      <c r="D193" s="24" t="inlineStr">
-        <is>
-          <t>algorithm</t>
-        </is>
-      </c>
-      <c r="E193" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/algorithm.py</t>
+      <c r="B193" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C193" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 3 – Data types in python</t>
+        </is>
+      </c>
+      <c r="D193" s="22" t="inlineStr">
+        <is>
+          <t>data-types</t>
+        </is>
+      </c>
+      <c r="E193" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/data-types.py</t>
+        </is>
+      </c>
+      <c r="F193" s="22" t="inlineStr">
+        <is>
+          <t>M1L3 Activity 1: Data types</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="24" t="inlineStr">
+      <c r="A194" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B194" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C194" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
-        </is>
-      </c>
-      <c r="D194" s="24" t="inlineStr">
-        <is>
-          <t>flowchart</t>
-        </is>
-      </c>
-      <c r="E194" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/flowchart.py</t>
+      <c r="B194" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C194" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 3 – Data types in python</t>
+        </is>
+      </c>
+      <c r="D194" s="22" t="inlineStr">
+        <is>
+          <t>typecasting</t>
+        </is>
+      </c>
+      <c r="E194" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/typecasting.py</t>
+        </is>
+      </c>
+      <c r="F194" s="22" t="inlineStr">
+        <is>
+          <t>M1L3 Activity 2: Typecasting</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="24" t="inlineStr">
+      <c r="A195" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B195" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C195" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 1 – Setting Up Dev Tools &amp; Intro to Python</t>
-        </is>
-      </c>
-      <c r="D195" s="24" t="inlineStr">
-        <is>
-          <t>platform-introduction</t>
-        </is>
-      </c>
-      <c r="E195" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-01/platform-introduction.py</t>
+      <c r="B195" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C195" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 3 – Data types in python</t>
+        </is>
+      </c>
+      <c r="D195" s="22" t="inlineStr">
+        <is>
+          <t>string-operation</t>
+        </is>
+      </c>
+      <c r="E195" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/string-operation.py</t>
+        </is>
+      </c>
+      <c r="F195" s="22" t="inlineStr">
+        <is>
+          <t>M1L3 Activity 3: String operation</t>
         </is>
       </c>
     </row>
@@ -5856,103 +6104,123 @@
       </c>
       <c r="B196" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C196" s="24" t="inlineStr">
         <is>
-          <t>Lesson 2 – Getting started with programming</t>
+          <t>Lesson 3 – Data types in python</t>
         </is>
       </c>
       <c r="D196" s="24" t="inlineStr">
         <is>
-          <t>welcome-to-the-world-of-coding</t>
+          <t>congratulations-message</t>
         </is>
       </c>
       <c r="E196" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/welcome-to-the-world-of-coding.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/congratulations-message/congratulations-message.py</t>
+        </is>
+      </c>
+      <c r="F196" s="24" t="inlineStr">
+        <is>
+          <t>M1L3 ACP : Congratulations message</t>
         </is>
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="24" t="inlineStr">
+      <c r="A197" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B197" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C197" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 2 – Getting started with programming</t>
-        </is>
-      </c>
-      <c r="D197" s="24" t="inlineStr">
-        <is>
-          <t>understanding-the-variables</t>
-        </is>
-      </c>
-      <c r="E197" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/understanding-the-variables.py</t>
+      <c r="B197" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C197" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 4 – Python Operators – I</t>
+        </is>
+      </c>
+      <c r="D197" s="22" t="inlineStr">
+        <is>
+          <t>average</t>
+        </is>
+      </c>
+      <c r="E197" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/average.py</t>
+        </is>
+      </c>
+      <c r="F197" s="22" t="inlineStr">
+        <is>
+          <t>M1L4 Activity 1: Average</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="24" t="inlineStr">
+      <c r="A198" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B198" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C198" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 2 – Getting started with programming</t>
-        </is>
-      </c>
-      <c r="D198" s="24" t="inlineStr">
-        <is>
-          <t>keywords</t>
-        </is>
-      </c>
-      <c r="E198" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-02/keywords.py</t>
+      <c r="B198" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C198" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 4 – Python Operators – I</t>
+        </is>
+      </c>
+      <c r="D198" s="22" t="inlineStr">
+        <is>
+          <t>count-the-notes</t>
+        </is>
+      </c>
+      <c r="E198" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/count-the-notes.py</t>
+        </is>
+      </c>
+      <c r="F198" s="22" t="inlineStr">
+        <is>
+          <t>M1L4 Activity 2: Count the notes</t>
         </is>
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="24" t="inlineStr">
+      <c r="A199" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B199" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C199" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 3 – Data types in python</t>
-        </is>
-      </c>
-      <c r="D199" s="24" t="inlineStr">
-        <is>
-          <t>data-types</t>
-        </is>
-      </c>
-      <c r="E199" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/data-types.py</t>
+      <c r="B199" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C199" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 4 – Python Operators – I</t>
+        </is>
+      </c>
+      <c r="D199" s="22" t="inlineStr">
+        <is>
+          <t>percentage-calculation</t>
+        </is>
+      </c>
+      <c r="E199" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/percentage-calculation.py</t>
+        </is>
+      </c>
+      <c r="F199" s="22" t="inlineStr">
+        <is>
+          <t>M1L4 Activity 3: Percentage calculation</t>
         </is>
       </c>
     </row>
@@ -5964,130 +6232,155 @@
       </c>
       <c r="B200" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C200" s="24" t="inlineStr">
         <is>
-          <t>Lesson 3 – Data types in python</t>
+          <t>Lesson 4 – Python Operators – I</t>
         </is>
       </c>
       <c r="D200" s="24" t="inlineStr">
         <is>
-          <t>typecasting</t>
+          <t>square-root</t>
         </is>
       </c>
       <c r="E200" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/typecasting.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/square-root/square-root.py</t>
+        </is>
+      </c>
+      <c r="F200" s="24" t="inlineStr">
+        <is>
+          <t>M1L4 ACP: Square root</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="24" t="inlineStr">
+      <c r="A201" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B201" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C201" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 3 – Data types in python</t>
-        </is>
-      </c>
-      <c r="D201" s="24" t="inlineStr">
-        <is>
-          <t>string-operation</t>
-        </is>
-      </c>
-      <c r="E201" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-03/string-operation.py</t>
+      <c r="B201" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C201" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D201" s="22" t="inlineStr">
+        <is>
+          <t>conditional-statements</t>
+        </is>
+      </c>
+      <c r="E201" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/conditional-statements.py</t>
+        </is>
+      </c>
+      <c r="F201" s="22" t="inlineStr">
+        <is>
+          <t>M1L5 Activity 1: Conditional statements</t>
         </is>
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="24" t="inlineStr">
+      <c r="A202" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B202" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C202" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 4 – Python Operators – I</t>
-        </is>
-      </c>
-      <c r="D202" s="24" t="inlineStr">
-        <is>
-          <t>average</t>
-        </is>
-      </c>
-      <c r="E202" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/average.py</t>
+      <c r="B202" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C202" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D202" s="22" t="inlineStr">
+        <is>
+          <t>profit-loss</t>
+        </is>
+      </c>
+      <c r="E202" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/profit-loss.py</t>
+        </is>
+      </c>
+      <c r="F202" s="22" t="inlineStr">
+        <is>
+          <t>M1L5 Activity 2: Profit loss</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="24" t="inlineStr">
+      <c r="A203" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B203" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C203" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 4 – Python Operators – I</t>
-        </is>
-      </c>
-      <c r="D203" s="24" t="inlineStr">
-        <is>
-          <t>count-the-notes</t>
-        </is>
-      </c>
-      <c r="E203" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/count-the-notes.py</t>
+      <c r="B203" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C203" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D203" s="22" t="inlineStr">
+        <is>
+          <t>checking-the-number-greater-or-smaller</t>
+        </is>
+      </c>
+      <c r="E203" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/checking-the-number-greater-or-smaller.py</t>
+        </is>
+      </c>
+      <c r="F203" s="22" t="inlineStr">
+        <is>
+          <t>M1L5 Activity 3: Checking the number greater or smaller</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="24" t="inlineStr">
+      <c r="A204" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B204" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C204" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 4 – Python Operators – I</t>
-        </is>
-      </c>
-      <c r="D204" s="24" t="inlineStr">
-        <is>
-          <t>percentage-calculation</t>
-        </is>
-      </c>
-      <c r="E204" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-04/percentage-calculation.py</t>
+      <c r="B204" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C204" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 5 – Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D204" s="22" t="inlineStr">
+        <is>
+          <t>odd-even</t>
+        </is>
+      </c>
+      <c r="E204" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/odd-even.py</t>
+        </is>
+      </c>
+      <c r="F204" s="22" t="inlineStr">
+        <is>
+          <t>M1L5 Activity 4: Odd-even</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6392,7 @@
       </c>
       <c r="B205" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C205" s="24" t="inlineStr">
@@ -6109,93 +6402,113 @@
       </c>
       <c r="D205" s="24" t="inlineStr">
         <is>
-          <t>conditional-statements</t>
+          <t>summer-times</t>
         </is>
       </c>
       <c r="E205" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/conditional-statements.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/summer-times/summer-times.py</t>
+        </is>
+      </c>
+      <c r="F205" s="24" t="inlineStr">
+        <is>
+          <t>M1L5 ACP : Summer times</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="24" t="inlineStr">
+      <c r="A206" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B206" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C206" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 5 – Conditional Statements</t>
-        </is>
-      </c>
-      <c r="D206" s="24" t="inlineStr">
-        <is>
-          <t>profit-loss</t>
-        </is>
-      </c>
-      <c r="E206" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/profit-loss.py</t>
+      <c r="B206" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C206" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D206" s="22" t="inlineStr">
+        <is>
+          <t>and-or-operator</t>
+        </is>
+      </c>
+      <c r="E206" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/and-or-operator.py</t>
+        </is>
+      </c>
+      <c r="F206" s="22" t="inlineStr">
+        <is>
+          <t>M1L6 Activity 1: AND-OR operator</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="24" t="inlineStr">
+      <c r="A207" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B207" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C207" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 5 – Conditional Statements</t>
-        </is>
-      </c>
-      <c r="D207" s="24" t="inlineStr">
-        <is>
-          <t>checking-the-number-greater-or-smaller</t>
-        </is>
-      </c>
-      <c r="E207" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/checking-the-number-greater-or-smaller.py</t>
+      <c r="B207" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C207" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D207" s="22" t="inlineStr">
+        <is>
+          <t>not-equal-operator</t>
+        </is>
+      </c>
+      <c r="E207" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/not-equal-operator.py</t>
+        </is>
+      </c>
+      <c r="F207" s="22" t="inlineStr">
+        <is>
+          <t>M1L6 Activity 2: NOT Equal Operator</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="24" t="inlineStr">
+      <c r="A208" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B208" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C208" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 5 – Conditional Statements</t>
-        </is>
-      </c>
-      <c r="D208" s="24" t="inlineStr">
-        <is>
-          <t>odd-even</t>
-        </is>
-      </c>
-      <c r="E208" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-05/odd-even.py</t>
+      <c r="B208" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C208" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 6 – Python Operator II</t>
+        </is>
+      </c>
+      <c r="D208" s="22" t="inlineStr">
+        <is>
+          <t>bmi-checker</t>
+        </is>
+      </c>
+      <c r="E208" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/bmi-checker.py</t>
+        </is>
+      </c>
+      <c r="F208" s="22" t="inlineStr">
+        <is>
+          <t>M1L6 Activity 3: BMI Checker</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6520,7 @@
       </c>
       <c r="B209" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C209" s="24" t="inlineStr">
@@ -6217,93 +6530,113 @@
       </c>
       <c r="D209" s="24" t="inlineStr">
         <is>
-          <t>and-or-operator</t>
+          <t>checking-alphabets</t>
         </is>
       </c>
       <c r="E209" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/and-or-operator.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/checking-alphabets/checking-alphabets.py</t>
+        </is>
+      </c>
+      <c r="F209" s="24" t="inlineStr">
+        <is>
+          <t>M1L6 ACP: Checking Alphabets</t>
         </is>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="24" t="inlineStr">
+      <c r="A210" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B210" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C210" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 6 – Python Operator II</t>
-        </is>
-      </c>
-      <c r="D210" s="24" t="inlineStr">
-        <is>
-          <t>not-equal-operator</t>
-        </is>
-      </c>
-      <c r="E210" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/not-equal-operator.py</t>
+      <c r="B210" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C210" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Python Operators III</t>
+        </is>
+      </c>
+      <c r="D210" s="22" t="inlineStr">
+        <is>
+          <t>identity-operator</t>
+        </is>
+      </c>
+      <c r="E210" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/identity-operator.py</t>
+        </is>
+      </c>
+      <c r="F210" s="22" t="inlineStr">
+        <is>
+          <t>M1L7 Activity 1: Identity operator</t>
         </is>
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="24" t="inlineStr">
+      <c r="A211" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B211" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C211" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 6 – Python Operator II</t>
-        </is>
-      </c>
-      <c r="D211" s="24" t="inlineStr">
-        <is>
-          <t>bmi-checker</t>
-        </is>
-      </c>
-      <c r="E211" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-06/bmi-checker.py</t>
+      <c r="B211" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C211" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 7 – Python Operators III</t>
+        </is>
+      </c>
+      <c r="D211" s="22" t="inlineStr">
+        <is>
+          <t>bitwise-operator</t>
+        </is>
+      </c>
+      <c r="E211" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/bitwise-operator.py</t>
+        </is>
+      </c>
+      <c r="F211" s="22" t="inlineStr">
+        <is>
+          <t>M1L7 Activity 2: Bitwise operator</t>
         </is>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="24" t="inlineStr">
+      <c r="A212" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B212" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C212" s="24" t="inlineStr">
+      <c r="B212" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C212" s="22" t="inlineStr">
         <is>
           <t>Lesson 7 – Python Operators III</t>
         </is>
       </c>
-      <c r="D212" s="24" t="inlineStr">
-        <is>
-          <t>identity-operator</t>
-        </is>
-      </c>
-      <c r="E212" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/identity-operator.py</t>
+      <c r="D212" s="22" t="inlineStr">
+        <is>
+          <t>grading-system</t>
+        </is>
+      </c>
+      <c r="E212" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/grading-system.py</t>
+        </is>
+      </c>
+      <c r="F212" s="22" t="inlineStr">
+        <is>
+          <t>M1L7 Activity 3: Grading system</t>
         </is>
       </c>
     </row>
@@ -6315,7 +6648,7 @@
       </c>
       <c r="B213" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C213" s="24" t="inlineStr">
@@ -6325,120 +6658,145 @@
       </c>
       <c r="D213" s="24" t="inlineStr">
         <is>
-          <t>bitwise-operator</t>
+          <t>ascii-value</t>
         </is>
       </c>
       <c r="E213" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/bitwise-operator.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/ascii-value/ascii-value.py</t>
+        </is>
+      </c>
+      <c r="F213" s="24" t="inlineStr">
+        <is>
+          <t>M1L7 ACP: ASCII value</t>
         </is>
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="24" t="inlineStr">
+      <c r="A214" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B214" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C214" s="24" t="inlineStr">
-        <is>
-          <t>Lesson 7 – Python Operators III</t>
-        </is>
-      </c>
-      <c r="D214" s="24" t="inlineStr">
-        <is>
-          <t>grading-system</t>
-        </is>
-      </c>
-      <c r="E214" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-07/grading-system.py</t>
+      <c r="B214" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C214" s="22" t="inlineStr">
+        <is>
+          <t>Lesson 8 – Python challenge</t>
+        </is>
+      </c>
+      <c r="D214" s="22" t="inlineStr">
+        <is>
+          <t>operator-precedence</t>
+        </is>
+      </c>
+      <c r="E214" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/operator-precedence.py</t>
+        </is>
+      </c>
+      <c r="F214" s="22" t="inlineStr">
+        <is>
+          <t>M1L8 Activity 1: Operator precedence</t>
         </is>
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="24" t="inlineStr">
+      <c r="A215" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B215" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C215" s="24" t="inlineStr">
+      <c r="B215" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C215" s="22" t="inlineStr">
         <is>
           <t>Lesson 8 – Python challenge</t>
         </is>
       </c>
-      <c r="D215" s="24" t="inlineStr">
-        <is>
-          <t>operator-precedence</t>
-        </is>
-      </c>
-      <c r="E215" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/operator-precedence.py</t>
+      <c r="D215" s="22" t="inlineStr">
+        <is>
+          <t>divisible-number</t>
+        </is>
+      </c>
+      <c r="E215" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/divisible-number.py</t>
+        </is>
+      </c>
+      <c r="F215" s="22" t="inlineStr">
+        <is>
+          <t>M1L8 Activity 2: Divisible Number</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="24" t="inlineStr">
+      <c r="A216" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B216" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C216" s="24" t="inlineStr">
+      <c r="B216" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C216" s="22" t="inlineStr">
         <is>
           <t>Lesson 8 – Python challenge</t>
         </is>
       </c>
-      <c r="D216" s="24" t="inlineStr">
-        <is>
-          <t>divisible-number</t>
-        </is>
-      </c>
-      <c r="E216" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/divisible-number.py</t>
+      <c r="D216" s="22" t="inlineStr">
+        <is>
+          <t>mean-value</t>
+        </is>
+      </c>
+      <c r="E216" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/mean-value.py</t>
+        </is>
+      </c>
+      <c r="F216" s="22" t="inlineStr">
+        <is>
+          <t>M1L8 Activity 3: Mean Value</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="24" t="inlineStr">
+      <c r="A217" s="22" t="inlineStr">
         <is>
           <t>PY-M1</t>
         </is>
       </c>
-      <c r="B217" s="24" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C217" s="24" t="inlineStr">
+      <c r="B217" s="22" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C217" s="22" t="inlineStr">
         <is>
           <t>Lesson 8 – Python challenge</t>
         </is>
       </c>
-      <c r="D217" s="24" t="inlineStr">
-        <is>
-          <t>mean-value</t>
-        </is>
-      </c>
-      <c r="E217" s="25" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/mean-value.py</t>
+      <c r="D217" s="22" t="inlineStr">
+        <is>
+          <t>average-speed</t>
+        </is>
+      </c>
+      <c r="E217" s="23" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/average-speed.py</t>
+        </is>
+      </c>
+      <c r="F217" s="22" t="inlineStr">
+        <is>
+          <t>M1L8 Activity 4: Average speed</t>
         </is>
       </c>
     </row>
@@ -6450,7 +6808,7 @@
       </c>
       <c r="B218" s="24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C218" s="24" t="inlineStr">
@@ -6460,12 +6818,17 @@
       </c>
       <c r="D218" s="24" t="inlineStr">
         <is>
-          <t>average-speed</t>
+          <t>number-swap</t>
         </is>
       </c>
       <c r="E218" s="25" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/activities/lesson-08/average-speed.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/assignments/number-swap/number-swap.py</t>
+        </is>
+      </c>
+      <c r="F218" s="24" t="inlineStr">
+        <is>
+          <t>M1L8 ACP: Number swap</t>
         </is>
       </c>
     </row>
@@ -6495,6 +6858,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-03/secret-agent-name-badge.py</t>
         </is>
       </c>
+      <c r="F219" s="26" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="26" t="inlineStr">
@@ -6522,6 +6886,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-04/farm-harvest-calculator.py</t>
         </is>
       </c>
+      <c r="F220" s="26" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="26" t="inlineStr">
@@ -6549,6 +6914,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-05/weather-outfit-picker.py</t>
         </is>
       </c>
+      <c r="F221" s="26" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="26" t="inlineStr">
@@ -6576,6 +6942,7 @@
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m1/projects/lesson-06/smart-school-day-planner.py</t>
         </is>
       </c>
+      <c r="F222" s="26" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Add python_m2 assignments, activities and ACPs
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +112,16 @@
         <fgColor rgb="00DCEDC8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B3E5FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -125,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -206,6 +216,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -573,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F222"/>
+  <dimension ref="A1:F246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6943,6 +6965,774 @@
         </is>
       </c>
       <c r="F222" s="26" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B223" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C223" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 9 – Nested Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D223" s="28" t="inlineStr">
+        <is>
+          <t>exam-eligibility-check</t>
+        </is>
+      </c>
+      <c r="E223" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-09/exam-eligibility-check.py</t>
+        </is>
+      </c>
+      <c r="F223" s="28" t="inlineStr">
+        <is>
+          <t>M2L1 Activity 1: Exam Eligibility Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B224" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C224" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 9 – Nested Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D224" s="28" t="inlineStr">
+        <is>
+          <t>electricity-bill</t>
+        </is>
+      </c>
+      <c r="E224" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-09/electricity-bill.py</t>
+        </is>
+      </c>
+      <c r="F224" s="28" t="inlineStr">
+        <is>
+          <t>M2L1 Activity 2: Electricity bill</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B225" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C225" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 9 – Nested Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D225" s="28" t="inlineStr">
+        <is>
+          <t>customise-your-ride</t>
+        </is>
+      </c>
+      <c r="E225" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-09/customise-your-ride.py</t>
+        </is>
+      </c>
+      <c r="F225" s="28" t="inlineStr">
+        <is>
+          <t>M2L1 Activity 3: Customise your ride</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="30" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B226" s="30" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C226" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 9 – Nested Conditional Statements</t>
+        </is>
+      </c>
+      <c r="D226" s="30" t="inlineStr">
+        <is>
+          <t>check-age</t>
+        </is>
+      </c>
+      <c r="E226" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/assignments/check-age/check-age.py</t>
+        </is>
+      </c>
+      <c r="F226" s="30" t="inlineStr">
+        <is>
+          <t>M2L1 ACP : Check Age</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B227" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C227" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 10 – Loops</t>
+        </is>
+      </c>
+      <c r="D227" s="28" t="inlineStr">
+        <is>
+          <t>sum-of-whole-numbers</t>
+        </is>
+      </c>
+      <c r="E227" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-10/sum-of-whole-numbers.py</t>
+        </is>
+      </c>
+      <c r="F227" s="28" t="inlineStr">
+        <is>
+          <t>M2L2 Activity 1: Sum of whole numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B228" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C228" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 10 – Loops</t>
+        </is>
+      </c>
+      <c r="D228" s="28" t="inlineStr">
+        <is>
+          <t>reverse-a-string</t>
+        </is>
+      </c>
+      <c r="E228" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-10/reverse-a-string.py</t>
+        </is>
+      </c>
+      <c r="F228" s="28" t="inlineStr">
+        <is>
+          <t>M2L2 Activity 2: Reverse a String</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B229" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C229" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 10 – Loops</t>
+        </is>
+      </c>
+      <c r="D229" s="28" t="inlineStr">
+        <is>
+          <t>reverse-order</t>
+        </is>
+      </c>
+      <c r="E229" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-10/reverse-order.py</t>
+        </is>
+      </c>
+      <c r="F229" s="28" t="inlineStr">
+        <is>
+          <t>M2L2 Activity 3: reverse order</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="30" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B230" s="30" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C230" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 10 – Loops</t>
+        </is>
+      </c>
+      <c r="D230" s="30" t="inlineStr">
+        <is>
+          <t>power-calculator</t>
+        </is>
+      </c>
+      <c r="E230" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/assignments/power-calculator/power-calculator.py</t>
+        </is>
+      </c>
+      <c r="F230" s="30" t="inlineStr">
+        <is>
+          <t>M2L2 ACP : Power calculator</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B231" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C231" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 11 – While loop</t>
+        </is>
+      </c>
+      <c r="D231" s="28" t="inlineStr">
+        <is>
+          <t>sum-of-natural-numbers</t>
+        </is>
+      </c>
+      <c r="E231" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-11/sum-of-natural-numbers.py</t>
+        </is>
+      </c>
+      <c r="F231" s="28" t="inlineStr">
+        <is>
+          <t>M2L3 Activity 1: Sum of Natural Numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B232" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C232" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 11 – While loop</t>
+        </is>
+      </c>
+      <c r="D232" s="28" t="inlineStr">
+        <is>
+          <t>infinity</t>
+        </is>
+      </c>
+      <c r="E232" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-11/infinity.py</t>
+        </is>
+      </c>
+      <c r="F232" s="28" t="inlineStr">
+        <is>
+          <t>M2L3 Activity 2: Infinity</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B233" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C233" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 11 – While loop</t>
+        </is>
+      </c>
+      <c r="D233" s="28" t="inlineStr">
+        <is>
+          <t>armstrong-number</t>
+        </is>
+      </c>
+      <c r="E233" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-11/armstrong-number.py</t>
+        </is>
+      </c>
+      <c r="F233" s="28" t="inlineStr">
+        <is>
+          <t>M2L3 Activity 3: Armstrong number</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="30" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B234" s="30" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C234" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 11 – While loop</t>
+        </is>
+      </c>
+      <c r="D234" s="30" t="inlineStr">
+        <is>
+          <t>reverse-order</t>
+        </is>
+      </c>
+      <c r="E234" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/assignments/reverse-order/reverse-order.py</t>
+        </is>
+      </c>
+      <c r="F234" s="30" t="inlineStr">
+        <is>
+          <t>M2L3 ACP : Reverse order</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B235" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C235" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 12 – Nested loop</t>
+        </is>
+      </c>
+      <c r="D235" s="28" t="inlineStr">
+        <is>
+          <t>character-occurrence</t>
+        </is>
+      </c>
+      <c r="E235" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-12/character-occurrence.py</t>
+        </is>
+      </c>
+      <c r="F235" s="28" t="inlineStr">
+        <is>
+          <t>M2L4 Activity 1: Character occurrence</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B236" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C236" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 12 – Nested loop</t>
+        </is>
+      </c>
+      <c r="D236" s="28" t="inlineStr">
+        <is>
+          <t>is-this-a-prime-number</t>
+        </is>
+      </c>
+      <c r="E236" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-12/is-this-a-prime-number.py</t>
+        </is>
+      </c>
+      <c r="F236" s="28" t="inlineStr">
+        <is>
+          <t>M2L4 Activity 2: Is this a Prime Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B237" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C237" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 12 – Nested loop</t>
+        </is>
+      </c>
+      <c r="D237" s="28" t="inlineStr">
+        <is>
+          <t>mid-product</t>
+        </is>
+      </c>
+      <c r="E237" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-12/mid-product.py</t>
+        </is>
+      </c>
+      <c r="F237" s="28" t="inlineStr">
+        <is>
+          <t>M2L4 Activity 3: Mid product</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="30" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B238" s="30" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C238" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 12 – Nested loop</t>
+        </is>
+      </c>
+      <c r="D238" s="30" t="inlineStr">
+        <is>
+          <t>binary-conversion</t>
+        </is>
+      </c>
+      <c r="E238" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/assignments/binary-conversion/binary-conversion.py</t>
+        </is>
+      </c>
+      <c r="F238" s="30" t="inlineStr">
+        <is>
+          <t>M2L4 ACP: Binary conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B239" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C239" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 13 – Patterns</t>
+        </is>
+      </c>
+      <c r="D239" s="28" t="inlineStr">
+        <is>
+          <t>right-angle-triangle</t>
+        </is>
+      </c>
+      <c r="E239" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-13/right-angle-triangle.py</t>
+        </is>
+      </c>
+      <c r="F239" s="28" t="inlineStr">
+        <is>
+          <t>M2L5 Activity 1: Right angle triangle</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B240" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C240" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 13 – Patterns</t>
+        </is>
+      </c>
+      <c r="D240" s="28" t="inlineStr">
+        <is>
+          <t>floyds-triangle</t>
+        </is>
+      </c>
+      <c r="E240" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-13/floyds-triangle.py</t>
+        </is>
+      </c>
+      <c r="F240" s="28" t="inlineStr">
+        <is>
+          <t>M2L5 Activity 2: Floyd's triangle</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B241" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C241" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 13 – Patterns</t>
+        </is>
+      </c>
+      <c r="D241" s="28" t="inlineStr">
+        <is>
+          <t>diamond-pattern</t>
+        </is>
+      </c>
+      <c r="E241" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-13/diamond-pattern.py</t>
+        </is>
+      </c>
+      <c r="F241" s="28" t="inlineStr">
+        <is>
+          <t>M2L5 Activity 3: Diamond Pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="30" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B242" s="30" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C242" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 13 – Patterns</t>
+        </is>
+      </c>
+      <c r="D242" s="30" t="inlineStr">
+        <is>
+          <t>mirrored-triangle</t>
+        </is>
+      </c>
+      <c r="E242" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/assignments/mirrored-triangle/mirrored-triangle.py</t>
+        </is>
+      </c>
+      <c r="F242" s="30" t="inlineStr">
+        <is>
+          <t>M2L5 ACP : Mirrored Triangle</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B243" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C243" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 14 – Introduction to Turtle</t>
+        </is>
+      </c>
+      <c r="D243" s="28" t="inlineStr">
+        <is>
+          <t>polygon</t>
+        </is>
+      </c>
+      <c r="E243" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-14/polygon.py</t>
+        </is>
+      </c>
+      <c r="F243" s="28" t="inlineStr">
+        <is>
+          <t>M2L6 Activity 1: Polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B244" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C244" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 14 – Introduction to Turtle</t>
+        </is>
+      </c>
+      <c r="D244" s="28" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="E244" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-14/star.py</t>
+        </is>
+      </c>
+      <c r="F244" s="28" t="inlineStr">
+        <is>
+          <t>M2L6 Activity 2: Star</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="28" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B245" s="28" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C245" s="28" t="inlineStr">
+        <is>
+          <t>Lesson 14 – Introduction to Turtle</t>
+        </is>
+      </c>
+      <c r="D245" s="28" t="inlineStr">
+        <is>
+          <t>spiral-pattern</t>
+        </is>
+      </c>
+      <c r="E245" s="29" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/activities/lesson-14/spiral-pattern.py</t>
+        </is>
+      </c>
+      <c r="F245" s="28" t="inlineStr">
+        <is>
+          <t>M2L6 Activity 3: Spiral pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="30" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B246" s="30" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C246" s="30" t="inlineStr">
+        <is>
+          <t>Lesson 14 – Introduction to Turtle</t>
+        </is>
+      </c>
+      <c r="D246" s="30" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="E246" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/assignments/square/square.py</t>
+        </is>
+      </c>
+      <c r="F246" s="30" t="inlineStr">
+        <is>
+          <t>M2L6 ACP: Square</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -7167,6 +7957,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E220" r:id="rId219"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E221" r:id="rId220"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId245"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add python_m2 lesson-plan projects not on the submission form
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -122,6 +122,11 @@
         <fgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -135,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -228,6 +233,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -595,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F246"/>
+  <dimension ref="A1:F248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7733,6 +7744,62 @@
           <t>M2L6 ACP: Square</t>
         </is>
       </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="32" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B247" s="32" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C247" s="32" t="inlineStr">
+        <is>
+          <t>Lesson 11 – While loop</t>
+        </is>
+      </c>
+      <c r="D247" s="32" t="inlineStr">
+        <is>
+          <t>my-chore-checklist-countdown</t>
+        </is>
+      </c>
+      <c r="E247" s="33" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/projects/lesson-11/my-chore-checklist-countdown.py</t>
+        </is>
+      </c>
+      <c r="F247" s="32" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="32" t="inlineStr">
+        <is>
+          <t>PY-M2</t>
+        </is>
+      </c>
+      <c r="B248" s="32" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C248" s="32" t="inlineStr">
+        <is>
+          <t>Lesson 12 – Nested loop</t>
+        </is>
+      </c>
+      <c r="D248" s="32" t="inlineStr">
+        <is>
+          <t>atm-cash-dispenser</t>
+        </is>
+      </c>
+      <c r="E248" s="33" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m2/projects/lesson-12/atm-cash-dispenser.py</t>
+        </is>
+      </c>
+      <c r="F248" s="32" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -7981,6 +8048,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E244" r:id="rId243"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E245" r:id="rId244"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E248" r:id="rId247"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Python M3 Functions and Modules activities, ACPs and projects
Keyed to the M3 Activity & ACP submission form, in form order.
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -127,6 +127,21 @@
         <fgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCBC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1C4E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B2DFDB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -140,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -239,6 +254,24 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -606,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F248"/>
+  <dimension ref="A1:F274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7800,6 +7833,830 @@
         </is>
       </c>
       <c r="F248" s="32" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B249" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C249" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 15 – Function</t>
+        </is>
+      </c>
+      <c r="D249" s="34" t="inlineStr">
+        <is>
+          <t>well-wishes</t>
+        </is>
+      </c>
+      <c r="E249" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-15/well-wishes.py</t>
+        </is>
+      </c>
+      <c r="F249" s="34" t="inlineStr">
+        <is>
+          <t>M3L1 Activity 1: Well wishes</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B250" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C250" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 15 – Function</t>
+        </is>
+      </c>
+      <c r="D250" s="34" t="inlineStr">
+        <is>
+          <t>weather-condition</t>
+        </is>
+      </c>
+      <c r="E250" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-15/weather-condition.py</t>
+        </is>
+      </c>
+      <c r="F250" s="34" t="inlineStr">
+        <is>
+          <t>M3L1 Activity 2: Weather condition</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B251" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C251" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 15 – Function</t>
+        </is>
+      </c>
+      <c r="D251" s="34" t="inlineStr">
+        <is>
+          <t>calculator</t>
+        </is>
+      </c>
+      <c r="E251" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-15/calculator.py</t>
+        </is>
+      </c>
+      <c r="F251" s="34" t="inlineStr">
+        <is>
+          <t>M3L1 Activity 3: Calculator</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="36" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B252" s="36" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C252" s="36" t="inlineStr">
+        <is>
+          <t>Lesson 15 – Function</t>
+        </is>
+      </c>
+      <c r="D252" s="36" t="inlineStr">
+        <is>
+          <t>circumference</t>
+        </is>
+      </c>
+      <c r="E252" s="37" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/assignments/circumference/circumference.py</t>
+        </is>
+      </c>
+      <c r="F252" s="36" t="inlineStr">
+        <is>
+          <t>M3L1 ACP : Circumference</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B253" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C253" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 16 – Arguments</t>
+        </is>
+      </c>
+      <c r="D253" s="34" t="inlineStr">
+        <is>
+          <t>sum-of-whole-numbers</t>
+        </is>
+      </c>
+      <c r="E253" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-16/sum-of-whole-numbers.py</t>
+        </is>
+      </c>
+      <c r="F253" s="34" t="inlineStr">
+        <is>
+          <t>M3L2 Activity 1: Sum of whole numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B254" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C254" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 16 – Arguments</t>
+        </is>
+      </c>
+      <c r="D254" s="34" t="inlineStr">
+        <is>
+          <t>cube-of-the-cube</t>
+        </is>
+      </c>
+      <c r="E254" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-16/cube-of-the-cube.py</t>
+        </is>
+      </c>
+      <c r="F254" s="34" t="inlineStr">
+        <is>
+          <t>M3L2 Activity 2: Cube of the cube</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B255" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C255" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 16 – Arguments</t>
+        </is>
+      </c>
+      <c r="D255" s="34" t="inlineStr">
+        <is>
+          <t>factorial</t>
+        </is>
+      </c>
+      <c r="E255" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-16/factorial.py</t>
+        </is>
+      </c>
+      <c r="F255" s="34" t="inlineStr">
+        <is>
+          <t>M3L2 Activity 3: Factorial</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="36" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B256" s="36" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C256" s="36" t="inlineStr">
+        <is>
+          <t>Lesson 16 – Arguments</t>
+        </is>
+      </c>
+      <c r="D256" s="36" t="inlineStr">
+        <is>
+          <t>shutdown</t>
+        </is>
+      </c>
+      <c r="E256" s="37" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/assignments/shutdown/shutdown.py</t>
+        </is>
+      </c>
+      <c r="F256" s="36" t="inlineStr">
+        <is>
+          <t>M3L2 ACP : Shutdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B257" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C257" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 17 – Keywords</t>
+        </is>
+      </c>
+      <c r="D257" s="34" t="inlineStr">
+        <is>
+          <t>break</t>
+        </is>
+      </c>
+      <c r="E257" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-17/break.py</t>
+        </is>
+      </c>
+      <c r="F257" s="34" t="inlineStr">
+        <is>
+          <t>M3L3 Activity 1: Break</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B258" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C258" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 17 – Keywords</t>
+        </is>
+      </c>
+      <c r="D258" s="34" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="E258" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-17/pass.py</t>
+        </is>
+      </c>
+      <c r="F258" s="34" t="inlineStr">
+        <is>
+          <t>M3L3 Activity 2: Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B259" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C259" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 17 – Keywords</t>
+        </is>
+      </c>
+      <c r="D259" s="34" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="E259" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-17/continue.py</t>
+        </is>
+      </c>
+      <c r="F259" s="34" t="inlineStr">
+        <is>
+          <t>M3L3 Activity 3: Continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="36" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B260" s="36" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C260" s="36" t="inlineStr">
+        <is>
+          <t>Lesson 17 – Keywords</t>
+        </is>
+      </c>
+      <c r="D260" s="36" t="inlineStr">
+        <is>
+          <t>due-amount</t>
+        </is>
+      </c>
+      <c r="E260" s="37" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/assignments/due-amount/due-amount.py</t>
+        </is>
+      </c>
+      <c r="F260" s="36" t="inlineStr">
+        <is>
+          <t>M3L3 ACP : Due Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B261" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C261" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 18 – Exception Handling</t>
+        </is>
+      </c>
+      <c r="D261" s="34" t="inlineStr">
+        <is>
+          <t>value-error</t>
+        </is>
+      </c>
+      <c r="E261" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-18/value-error.py</t>
+        </is>
+      </c>
+      <c r="F261" s="34" t="inlineStr">
+        <is>
+          <t>M3L4 Activity 1: Value Error</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B262" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C262" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 18 – Exception Handling</t>
+        </is>
+      </c>
+      <c r="D262" s="34" t="inlineStr">
+        <is>
+          <t>multiple-exceptions</t>
+        </is>
+      </c>
+      <c r="E262" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-18/multiple-exceptions.py</t>
+        </is>
+      </c>
+      <c r="F262" s="34" t="inlineStr">
+        <is>
+          <t>M3L4 Activity 2: Multiple exceptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B263" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C263" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 18 – Exception Handling</t>
+        </is>
+      </c>
+      <c r="D263" s="34" t="inlineStr">
+        <is>
+          <t>bye-bye</t>
+        </is>
+      </c>
+      <c r="E263" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-18/bye-bye.py</t>
+        </is>
+      </c>
+      <c r="F263" s="34" t="inlineStr">
+        <is>
+          <t>M3L4 Activity 3: Bye Bye</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="36" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B264" s="36" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C264" s="36" t="inlineStr">
+        <is>
+          <t>Lesson 18 – Exception Handling</t>
+        </is>
+      </c>
+      <c r="D264" s="36" t="inlineStr">
+        <is>
+          <t>age-counter</t>
+        </is>
+      </c>
+      <c r="E264" s="37" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/assignments/age-counter/age-counter.py</t>
+        </is>
+      </c>
+      <c r="F264" s="36" t="inlineStr">
+        <is>
+          <t>M3L4 ACP: Age Counter</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B265" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C265" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 19 – Random and math module</t>
+        </is>
+      </c>
+      <c r="D265" s="34" t="inlineStr">
+        <is>
+          <t>number-game</t>
+        </is>
+      </c>
+      <c r="E265" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-19/number-game.py</t>
+        </is>
+      </c>
+      <c r="F265" s="34" t="inlineStr">
+        <is>
+          <t>M3L5 Activity 1: Number game</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B266" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C266" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 19 – Random and math module</t>
+        </is>
+      </c>
+      <c r="D266" s="34" t="inlineStr">
+        <is>
+          <t>rock-paper-scissors</t>
+        </is>
+      </c>
+      <c r="E266" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-19/rock-paper-scissors.py</t>
+        </is>
+      </c>
+      <c r="F266" s="34" t="inlineStr">
+        <is>
+          <t>M3L5 Activity 2: Rock paper scissors</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B267" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C267" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 19 – Random and math module</t>
+        </is>
+      </c>
+      <c r="D267" s="34" t="inlineStr">
+        <is>
+          <t>mathematical-operations</t>
+        </is>
+      </c>
+      <c r="E267" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-19/mathematical-operations.py</t>
+        </is>
+      </c>
+      <c r="F267" s="34" t="inlineStr">
+        <is>
+          <t>M3L5 Activity 3: Mathematical operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="36" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B268" s="36" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C268" s="36" t="inlineStr">
+        <is>
+          <t>Lesson 19 – Random and math module</t>
+        </is>
+      </c>
+      <c r="D268" s="36" t="inlineStr">
+        <is>
+          <t>trigonometric-value</t>
+        </is>
+      </c>
+      <c r="E268" s="37" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/assignments/trigonometric-value/trigonometric-value.py</t>
+        </is>
+      </c>
+      <c r="F268" s="36" t="inlineStr">
+        <is>
+          <t>M3L5 ACP : Trigonometric value</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B269" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C269" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 20 – Date, time, and calendar module</t>
+        </is>
+      </c>
+      <c r="D269" s="34" t="inlineStr">
+        <is>
+          <t>current-date-and-time</t>
+        </is>
+      </c>
+      <c r="E269" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-20/current-date-and-time.py</t>
+        </is>
+      </c>
+      <c r="F269" s="34" t="inlineStr">
+        <is>
+          <t>M3L6 Activity 1: Current date and time</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B270" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C270" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 20 – Date, time, and calendar module</t>
+        </is>
+      </c>
+      <c r="D270" s="34" t="inlineStr">
+        <is>
+          <t>random-date-and-time</t>
+        </is>
+      </c>
+      <c r="E270" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-20/random-date-and-time.py</t>
+        </is>
+      </c>
+      <c r="F270" s="34" t="inlineStr">
+        <is>
+          <t>M3L6 Activity 2: Random date and time</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="34" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B271" s="34" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C271" s="34" t="inlineStr">
+        <is>
+          <t>Lesson 20 – Date, time, and calendar module</t>
+        </is>
+      </c>
+      <c r="D271" s="34" t="inlineStr">
+        <is>
+          <t>trip-expenditure</t>
+        </is>
+      </c>
+      <c r="E271" s="35" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/activities/lesson-20/trip-expenditure.py</t>
+        </is>
+      </c>
+      <c r="F271" s="34" t="inlineStr">
+        <is>
+          <t>M3L6 Activity 3: Trip expenditure</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="36" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B272" s="36" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C272" s="36" t="inlineStr">
+        <is>
+          <t>Lesson 20 – Date, time, and calendar module</t>
+        </is>
+      </c>
+      <c r="D272" s="36" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="E272" s="37" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/assignments/months/months.py</t>
+        </is>
+      </c>
+      <c r="F272" s="36" t="inlineStr">
+        <is>
+          <t>M3L6 ACP: Months</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="38" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B273" s="38" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C273" s="38" t="inlineStr">
+        <is>
+          <t>Lesson 16 – Arguments</t>
+        </is>
+      </c>
+      <c r="D273" s="38" t="inlineStr">
+        <is>
+          <t>tip-the-waiter</t>
+        </is>
+      </c>
+      <c r="E273" s="39" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/projects/lesson-16/tip-the-waiter.py</t>
+        </is>
+      </c>
+      <c r="F273" s="38" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="38" t="inlineStr">
+        <is>
+          <t>PY-M3</t>
+        </is>
+      </c>
+      <c r="B274" s="38" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C274" s="38" t="inlineStr">
+        <is>
+          <t>Lesson 17 – Keywords</t>
+        </is>
+      </c>
+      <c r="D274" s="38" t="inlineStr">
+        <is>
+          <t>snack-vending-machine</t>
+        </is>
+      </c>
+      <c r="E274" s="39" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m3/projects/lesson-17/snack-vending-machine.py</t>
+        </is>
+      </c>
+      <c r="F274" s="38" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -8050,6 +8907,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId245"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E247" r:id="rId246"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E274" r:id="rId273"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Python M4 Data Structures activities, ACPs and projects
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -142,6 +142,21 @@
         <fgColor rgb="00B2DFDB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFECB3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C5CAE9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -155,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -272,6 +287,24 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -639,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F274"/>
+  <dimension ref="A1:F299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8657,6 +8690,798 @@
         </is>
       </c>
       <c r="F274" s="38" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B275" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C275" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 21 – Getting Started with Lists</t>
+        </is>
+      </c>
+      <c r="D275" s="40" t="inlineStr">
+        <is>
+          <t>lists</t>
+        </is>
+      </c>
+      <c r="E275" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-21/lists.py</t>
+        </is>
+      </c>
+      <c r="F275" s="40" t="inlineStr">
+        <is>
+          <t>M4L1 Activity 1: Lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B276" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C276" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 21 – Getting Started with Lists</t>
+        </is>
+      </c>
+      <c r="D276" s="40" t="inlineStr">
+        <is>
+          <t>word-matching</t>
+        </is>
+      </c>
+      <c r="E276" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-21/word-matching.py</t>
+        </is>
+      </c>
+      <c r="F276" s="40" t="inlineStr">
+        <is>
+          <t>M4L1 Activity 2: Word Matching</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B277" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C277" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 21 – Getting Started with Lists</t>
+        </is>
+      </c>
+      <c r="D277" s="40" t="inlineStr">
+        <is>
+          <t>play-with-lists</t>
+        </is>
+      </c>
+      <c r="E277" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-21/play-with-lists.py</t>
+        </is>
+      </c>
+      <c r="F277" s="40" t="inlineStr">
+        <is>
+          <t>M4L1 Activity 3: Play with Lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="42" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B278" s="42" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C278" s="42" t="inlineStr">
+        <is>
+          <t>Lesson 21 – Getting Started with Lists</t>
+        </is>
+      </c>
+      <c r="D278" s="42" t="inlineStr">
+        <is>
+          <t>square-it-out</t>
+        </is>
+      </c>
+      <c r="E278" s="43" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/assignments/square-it-out/square-it-out.py</t>
+        </is>
+      </c>
+      <c r="F278" s="42" t="inlineStr">
+        <is>
+          <t>M4L1 ACP : Square it Out!</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B279" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C279" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 22 – Tuples</t>
+        </is>
+      </c>
+      <c r="D279" s="40" t="inlineStr">
+        <is>
+          <t>tuple-operations</t>
+        </is>
+      </c>
+      <c r="E279" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-22/tuple-operations.py</t>
+        </is>
+      </c>
+      <c r="F279" s="40" t="inlineStr">
+        <is>
+          <t>M4L2 Activity 1: Tuple Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B280" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C280" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 22 – Tuples</t>
+        </is>
+      </c>
+      <c r="D280" s="40" t="inlineStr">
+        <is>
+          <t>flip-flop</t>
+        </is>
+      </c>
+      <c r="E280" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-22/flip-flop.py</t>
+        </is>
+      </c>
+      <c r="F280" s="40" t="inlineStr">
+        <is>
+          <t>M4L2 Activity 2: Flip Flop</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B281" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C281" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 22 – Tuples</t>
+        </is>
+      </c>
+      <c r="D281" s="40" t="inlineStr">
+        <is>
+          <t>weather-prediction</t>
+        </is>
+      </c>
+      <c r="E281" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-22/weather-prediction.py</t>
+        </is>
+      </c>
+      <c r="F281" s="40" t="inlineStr">
+        <is>
+          <t>M4L2 Activity 3: Weather Prediction</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="42" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B282" s="42" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C282" s="42" t="inlineStr">
+        <is>
+          <t>Lesson 22 – Tuples</t>
+        </is>
+      </c>
+      <c r="D282" s="42" t="inlineStr">
+        <is>
+          <t>tuple-product</t>
+        </is>
+      </c>
+      <c r="E282" s="43" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/assignments/tuple-product/tuple-product.py</t>
+        </is>
+      </c>
+      <c r="F282" s="42" t="inlineStr">
+        <is>
+          <t>M4L2 ACP : Tuple Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B283" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C283" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 23 – All About Dictionary</t>
+        </is>
+      </c>
+      <c r="D283" s="40" t="inlineStr">
+        <is>
+          <t>get-rid-of-the-duplicates</t>
+        </is>
+      </c>
+      <c r="E283" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-23/get-rid-of-the-duplicates.py</t>
+        </is>
+      </c>
+      <c r="F283" s="40" t="inlineStr">
+        <is>
+          <t>M4L3 Activity 1: Get rid of the duplicates</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B284" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C284" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 23 – All About Dictionary</t>
+        </is>
+      </c>
+      <c r="D284" s="40" t="inlineStr">
+        <is>
+          <t>check-the-frequency</t>
+        </is>
+      </c>
+      <c r="E284" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-23/check-the-frequency.py</t>
+        </is>
+      </c>
+      <c r="F284" s="40" t="inlineStr">
+        <is>
+          <t>M4L3 Activity 2: Check the frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B285" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C285" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 23 – All About Dictionary</t>
+        </is>
+      </c>
+      <c r="D285" s="40" t="inlineStr">
+        <is>
+          <t>get-the-country-code</t>
+        </is>
+      </c>
+      <c r="E285" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-23/get-the-country-code.py</t>
+        </is>
+      </c>
+      <c r="F285" s="40" t="inlineStr">
+        <is>
+          <t>M4L3 Activity 3: Get the country code</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="42" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B286" s="42" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C286" s="42" t="inlineStr">
+        <is>
+          <t>Lesson 23 – All About Dictionary</t>
+        </is>
+      </c>
+      <c r="D286" s="42" t="inlineStr">
+        <is>
+          <t>check-the-frequency</t>
+        </is>
+      </c>
+      <c r="E286" s="43" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/assignments/check-the-frequency/check-the-frequency.py</t>
+        </is>
+      </c>
+      <c r="F286" s="42" t="inlineStr">
+        <is>
+          <t>M4L3 ACP : Check the frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B287" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C287" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 24 – Sets and Arrays</t>
+        </is>
+      </c>
+      <c r="D287" s="40" t="inlineStr">
+        <is>
+          <t>operations-on-sets</t>
+        </is>
+      </c>
+      <c r="E287" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-24/operations-on-sets.py</t>
+        </is>
+      </c>
+      <c r="F287" s="40" t="inlineStr">
+        <is>
+          <t>M4L4 Activity 1: Operations on Sets</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B288" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C288" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 24 – Sets and Arrays</t>
+        </is>
+      </c>
+      <c r="D288" s="40" t="inlineStr">
+        <is>
+          <t>set-intersection</t>
+        </is>
+      </c>
+      <c r="E288" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-24/set-intersection.py</t>
+        </is>
+      </c>
+      <c r="F288" s="40" t="inlineStr">
+        <is>
+          <t>M4L4 Activity 2: Set Intersection</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B289" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C289" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 24 – Sets and Arrays</t>
+        </is>
+      </c>
+      <c r="D289" s="40" t="inlineStr">
+        <is>
+          <t>arrays</t>
+        </is>
+      </c>
+      <c r="E289" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-24/arrays.py</t>
+        </is>
+      </c>
+      <c r="F289" s="40" t="inlineStr">
+        <is>
+          <t>M4L4 Activity 3: Arrays</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="42" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B290" s="42" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C290" s="42" t="inlineStr">
+        <is>
+          <t>Lesson 24 – Sets and Arrays</t>
+        </is>
+      </c>
+      <c r="D290" s="42" t="inlineStr">
+        <is>
+          <t>set-symmetric-difference</t>
+        </is>
+      </c>
+      <c r="E290" s="43" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/assignments/set-symmetric-difference/set-symmetric-difference.py</t>
+        </is>
+      </c>
+      <c r="F290" s="42" t="inlineStr">
+        <is>
+          <t>M4L4 ACP: Set Symmetric Difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B291" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C291" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Advanced Python Functions</t>
+        </is>
+      </c>
+      <c r="D291" s="40" t="inlineStr">
+        <is>
+          <t>hands-on-map</t>
+        </is>
+      </c>
+      <c r="E291" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-25/hands-on-map.py</t>
+        </is>
+      </c>
+      <c r="F291" s="40" t="inlineStr">
+        <is>
+          <t>M4L5 Activity 1: Hands-on Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B292" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C292" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Advanced Python Functions</t>
+        </is>
+      </c>
+      <c r="D292" s="40" t="inlineStr">
+        <is>
+          <t>zip-it</t>
+        </is>
+      </c>
+      <c r="E292" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-25/zip-it.py</t>
+        </is>
+      </c>
+      <c r="F292" s="40" t="inlineStr">
+        <is>
+          <t>M4L5 Activity 2: Zip It!</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B293" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C293" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Advanced Python Functions</t>
+        </is>
+      </c>
+      <c r="D293" s="40" t="inlineStr">
+        <is>
+          <t>thats-the-exit</t>
+        </is>
+      </c>
+      <c r="E293" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-25/thats-the-exit.py</t>
+        </is>
+      </c>
+      <c r="F293" s="40" t="inlineStr">
+        <is>
+          <t>M4L5 Activity 3: That’s the exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="42" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B294" s="42" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C294" s="42" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Advanced Python Functions</t>
+        </is>
+      </c>
+      <c r="D294" s="42" t="inlineStr">
+        <is>
+          <t>list-comprehension-practice</t>
+        </is>
+      </c>
+      <c r="E294" s="43" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/assignments/list-comprehension-practice/list-comprehension-practice.py</t>
+        </is>
+      </c>
+      <c r="F294" s="42" t="inlineStr">
+        <is>
+          <t>M4L5 ACP : List Comprehension Practice</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B295" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C295" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Python Challenges</t>
+        </is>
+      </c>
+      <c r="D295" s="40" t="inlineStr">
+        <is>
+          <t>tic-tac-toe-game</t>
+        </is>
+      </c>
+      <c r="E295" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-26/tic-tac-toe-game.py</t>
+        </is>
+      </c>
+      <c r="F295" s="40" t="inlineStr">
+        <is>
+          <t>M4L6 Activity 1: Tic Tac Toe Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="40" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B296" s="40" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C296" s="40" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Python Challenges</t>
+        </is>
+      </c>
+      <c r="D296" s="40" t="inlineStr">
+        <is>
+          <t>guess-the-number-game</t>
+        </is>
+      </c>
+      <c r="E296" s="41" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/activities/lesson-26/guess-the-number-game.py</t>
+        </is>
+      </c>
+      <c r="F296" s="40" t="inlineStr">
+        <is>
+          <t>M4L6 Activity 2: Guess the Number Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="42" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B297" s="42" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C297" s="42" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Python Challenges</t>
+        </is>
+      </c>
+      <c r="D297" s="42" t="inlineStr">
+        <is>
+          <t>random-password-challenge</t>
+        </is>
+      </c>
+      <c r="E297" s="43" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/assignments/random-password-challenge/random-password-challenge.py</t>
+        </is>
+      </c>
+      <c r="F297" s="42" t="inlineStr">
+        <is>
+          <t>M4L6 ACP: Random Password Challenge</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="44" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B298" s="44" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C298" s="44" t="inlineStr">
+        <is>
+          <t>Lesson 24 – Sets and Arrays</t>
+        </is>
+      </c>
+      <c r="D298" s="44" t="inlineStr">
+        <is>
+          <t>class-fruit-basket-organizer</t>
+        </is>
+      </c>
+      <c r="E298" s="45" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/projects/lesson-24/class-fruit-basket-organizer.py</t>
+        </is>
+      </c>
+      <c r="F298" s="44" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="44" t="inlineStr">
+        <is>
+          <t>PY-M4</t>
+        </is>
+      </c>
+      <c r="B299" s="44" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C299" s="44" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Advanced Python Functions</t>
+        </is>
+      </c>
+      <c r="D299" s="44" t="inlineStr">
+        <is>
+          <t>school-store-inventory-checker</t>
+        </is>
+      </c>
+      <c r="E299" s="45" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m4/projects/lesson-25/school-store-inventory-checker.py</t>
+        </is>
+      </c>
+      <c r="F299" s="44" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -8933,6 +9758,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E272" r:id="rId271"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E273" r:id="rId272"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E299" r:id="rId298"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Python M5 Object-Oriented Programming activities and assignments
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="28">
     <fill>
       <patternFill/>
     </fill>
@@ -157,6 +157,21 @@
         <fgColor rgb="00FFCDD2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0080DEEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B39DDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AED581"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -170,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -305,6 +320,24 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -672,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F299"/>
+  <dimension ref="A1:F324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9482,6 +9515,802 @@
         </is>
       </c>
       <c r="F299" s="44" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B300" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C300" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D300" s="46" t="inlineStr">
+        <is>
+          <t>student-class</t>
+        </is>
+      </c>
+      <c r="E300" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-27/student-class.py</t>
+        </is>
+      </c>
+      <c r="F300" s="46" t="inlineStr">
+        <is>
+          <t>M5L1 Activity 1: Student Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B301" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C301" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D301" s="46" t="inlineStr">
+        <is>
+          <t>class-vehicle</t>
+        </is>
+      </c>
+      <c r="E301" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-27/class-vehicle.py</t>
+        </is>
+      </c>
+      <c r="F301" s="46" t="inlineStr">
+        <is>
+          <t>M5L1 Activity 2: Class Vehicle</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B302" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C302" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D302" s="46" t="inlineStr">
+        <is>
+          <t>class-parrot</t>
+        </is>
+      </c>
+      <c r="E302" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-27/class-parrot.py</t>
+        </is>
+      </c>
+      <c r="F302" s="46" t="inlineStr">
+        <is>
+          <t>M5L1 Activity 3: Class Parrot</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="48" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B303" s="48" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C303" s="48" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D303" s="48" t="inlineStr">
+        <is>
+          <t>dog-breed</t>
+        </is>
+      </c>
+      <c r="E303" s="49" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/assignments/dog-breed/dog-breed.py</t>
+        </is>
+      </c>
+      <c r="F303" s="48" t="inlineStr">
+        <is>
+          <t>M5L1 ACP : Dog Breed</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B304" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C304" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 28 – More on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D304" s="46" t="inlineStr">
+        <is>
+          <t>string-upper-case</t>
+        </is>
+      </c>
+      <c r="E304" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-28/string-upper-case.py</t>
+        </is>
+      </c>
+      <c r="F304" s="46" t="inlineStr">
+        <is>
+          <t>M5L2 Activity 1: String Upper Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B305" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C305" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 28 – More on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D305" s="46" t="inlineStr">
+        <is>
+          <t>employee-in-and-out</t>
+        </is>
+      </c>
+      <c r="E305" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-28/employee-in-and-out.py</t>
+        </is>
+      </c>
+      <c r="F305" s="46" t="inlineStr">
+        <is>
+          <t>M5L2 Activity 2: Employee in and Out</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B306" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C306" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 28 – More on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D306" s="46" t="inlineStr">
+        <is>
+          <t>pair-of-elements</t>
+        </is>
+      </c>
+      <c r="E306" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-28/pair-of-elements.py</t>
+        </is>
+      </c>
+      <c r="F306" s="46" t="inlineStr">
+        <is>
+          <t>M5L2 Activity 3: Pair of Elements</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="48" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B307" s="48" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C307" s="48" t="inlineStr">
+        <is>
+          <t>Lesson 28 – More on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D307" s="48" t="inlineStr">
+        <is>
+          <t>area-and-perimeter-of-circle</t>
+        </is>
+      </c>
+      <c r="E307" s="49" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/assignments/area-and-perimeter-of-circle/area-and-perimeter-of-circle.py</t>
+        </is>
+      </c>
+      <c r="F307" s="48" t="inlineStr">
+        <is>
+          <t>M5L2 ACP : Area and Perimeter of circle</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B308" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C308" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 29 – Inheritance</t>
+        </is>
+      </c>
+      <c r="D308" s="46" t="inlineStr">
+        <is>
+          <t>is-this-a-bus</t>
+        </is>
+      </c>
+      <c r="E308" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-29/is-this-a-bus.py</t>
+        </is>
+      </c>
+      <c r="F308" s="46" t="inlineStr">
+        <is>
+          <t>M5L3 Activity 1: Is this a bus?</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B309" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C309" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 29 – Inheritance</t>
+        </is>
+      </c>
+      <c r="D309" s="46" t="inlineStr">
+        <is>
+          <t>employee-inheritance</t>
+        </is>
+      </c>
+      <c r="E309" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-29/employee-inheritance.py</t>
+        </is>
+      </c>
+      <c r="F309" s="46" t="inlineStr">
+        <is>
+          <t>M5L3 Activity 2: Employee Inheritance</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B310" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C310" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 29 – Inheritance</t>
+        </is>
+      </c>
+      <c r="D310" s="46" t="inlineStr">
+        <is>
+          <t>super-penguin</t>
+        </is>
+      </c>
+      <c r="E310" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-29/super-penguin.py</t>
+        </is>
+      </c>
+      <c r="F310" s="46" t="inlineStr">
+        <is>
+          <t>M5L3 Activity 3: Super Penguin</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="48" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B311" s="48" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C311" s="48" t="inlineStr">
+        <is>
+          <t>Lesson 29 – Inheritance</t>
+        </is>
+      </c>
+      <c r="D311" s="48" t="inlineStr">
+        <is>
+          <t>bus-fare</t>
+        </is>
+      </c>
+      <c r="E311" s="49" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/assignments/bus-fare/bus-fare.py</t>
+        </is>
+      </c>
+      <c r="F311" s="48" t="inlineStr">
+        <is>
+          <t>M5L3 ACP : Bus Fare</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B312" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C312" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Encapsulation and Special Functions</t>
+        </is>
+      </c>
+      <c r="D312" s="46" t="inlineStr">
+        <is>
+          <t>keep-it-private</t>
+        </is>
+      </c>
+      <c r="E312" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-30/keep-it-private.py</t>
+        </is>
+      </c>
+      <c r="F312" s="46" t="inlineStr">
+        <is>
+          <t>M5L4 Activity 1: Keep It Private!</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B313" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C313" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Encapsulation and Special Functions</t>
+        </is>
+      </c>
+      <c r="D313" s="46" t="inlineStr">
+        <is>
+          <t>computer-price</t>
+        </is>
+      </c>
+      <c r="E313" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-30/computer-price.py</t>
+        </is>
+      </c>
+      <c r="F313" s="46" t="inlineStr">
+        <is>
+          <t>M5L4 Activity 2: Computer Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B314" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C314" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Encapsulation and Special Functions</t>
+        </is>
+      </c>
+      <c r="D314" s="46" t="inlineStr">
+        <is>
+          <t>point-function</t>
+        </is>
+      </c>
+      <c r="E314" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-30/point-function.py</t>
+        </is>
+      </c>
+      <c r="F314" s="46" t="inlineStr">
+        <is>
+          <t>M5L4 Activity 3: Point Function</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="48" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B315" s="48" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C315" s="48" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Encapsulation and Special Functions</t>
+        </is>
+      </c>
+      <c r="D315" s="48" t="inlineStr">
+        <is>
+          <t>class-string-reverse</t>
+        </is>
+      </c>
+      <c r="E315" s="49" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/assignments/class-string-reverse/class-string-reverse.py</t>
+        </is>
+      </c>
+      <c r="F315" s="48" t="inlineStr">
+        <is>
+          <t>M5L4 ACP: Class String Reverse</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B316" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C316" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Abstraction and Polymorphism</t>
+        </is>
+      </c>
+      <c r="D316" s="46" t="inlineStr">
+        <is>
+          <t>abstract-class</t>
+        </is>
+      </c>
+      <c r="E316" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-31/abstract-class.py</t>
+        </is>
+      </c>
+      <c r="F316" s="46" t="inlineStr">
+        <is>
+          <t>M5L5 Activity 1: Abstract Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B317" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C317" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Abstraction and Polymorphism</t>
+        </is>
+      </c>
+      <c r="D317" s="46" t="inlineStr">
+        <is>
+          <t>class-animal</t>
+        </is>
+      </c>
+      <c r="E317" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-31/class-animal.py</t>
+        </is>
+      </c>
+      <c r="F317" s="46" t="inlineStr">
+        <is>
+          <t>M5L5 Activity 2: Class Animal</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B318" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C318" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Abstraction and Polymorphism</t>
+        </is>
+      </c>
+      <c r="D318" s="46" t="inlineStr">
+        <is>
+          <t>all-about-countries</t>
+        </is>
+      </c>
+      <c r="E318" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-31/all-about-countries.py</t>
+        </is>
+      </c>
+      <c r="F318" s="46" t="inlineStr">
+        <is>
+          <t>M5L5 Activity 3: All about Countries</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="48" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B319" s="48" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C319" s="48" t="inlineStr">
+        <is>
+          <t>Lesson 31 – Abstraction and Polymorphism</t>
+        </is>
+      </c>
+      <c r="D319" s="48" t="inlineStr">
+        <is>
+          <t>vehicle-polymorphism</t>
+        </is>
+      </c>
+      <c r="E319" s="49" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/assignments/vehicle-polymorphism/vehicle-polymorphism.py</t>
+        </is>
+      </c>
+      <c r="F319" s="48" t="inlineStr">
+        <is>
+          <t>M5L5 ACP : Vehicle Polymorphism</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B320" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C320" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Challenges on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D320" s="46" t="inlineStr">
+        <is>
+          <t>overload-operators</t>
+        </is>
+      </c>
+      <c r="E320" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-32/overload-operators.py</t>
+        </is>
+      </c>
+      <c r="F320" s="46" t="inlineStr">
+        <is>
+          <t>M5L6 Activity 1: Overload Operators</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B321" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C321" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Challenges on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D321" s="46" t="inlineStr">
+        <is>
+          <t>flashcards</t>
+        </is>
+      </c>
+      <c r="E321" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-32/flashcards.py</t>
+        </is>
+      </c>
+      <c r="F321" s="46" t="inlineStr">
+        <is>
+          <t>M5L6 Activity 2: Flashcards</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="46" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B322" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C322" s="46" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Challenges on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D322" s="46" t="inlineStr">
+        <is>
+          <t>fruit-quiz</t>
+        </is>
+      </c>
+      <c r="E322" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/activities/lesson-32/fruit-quiz.py</t>
+        </is>
+      </c>
+      <c r="F322" s="46" t="inlineStr">
+        <is>
+          <t>M5L6 Activity 3: Fruit Quiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="48" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B323" s="48" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C323" s="48" t="inlineStr">
+        <is>
+          <t>Lesson 32 – Challenges on Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="D323" s="48" t="inlineStr">
+        <is>
+          <t>integer-to-roman</t>
+        </is>
+      </c>
+      <c r="E323" s="49" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/assignments/integer-to-roman/integer-to-roman.py</t>
+        </is>
+      </c>
+      <c r="F323" s="48" t="inlineStr">
+        <is>
+          <t>M5L6 ACP: Integer to Roman</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="50" t="inlineStr">
+        <is>
+          <t>PY-M5</t>
+        </is>
+      </c>
+      <c r="B324" s="50" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C324" s="50" t="inlineStr">
+        <is>
+          <t>Lesson 29 – Inheritance</t>
+        </is>
+      </c>
+      <c r="D324" s="50" t="inlineStr">
+        <is>
+          <t>my-family-trait-tree</t>
+        </is>
+      </c>
+      <c r="E324" s="51" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m5/projects/lesson-29/my-family-trait-tree.py</t>
+        </is>
+      </c>
+      <c r="F324" s="50" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9783,6 +10612,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId296"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E298" r:id="rId297"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E324" r:id="rId323"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Python M6 - Game Building with Pygame
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="28">
+  <fills count="30">
     <fill>
       <patternFill/>
     </fill>
@@ -172,6 +172,16 @@
         <fgColor rgb="00AED581"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C5E1A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8BBD0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -185,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -338,6 +348,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -705,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F324"/>
+  <dimension ref="A1:F339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10311,6 +10333,486 @@
         </is>
       </c>
       <c r="F324" s="50" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B325" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C325" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 33 – Let's Begin with Pygame</t>
+        </is>
+      </c>
+      <c r="D325" s="52" t="inlineStr">
+        <is>
+          <t>pygame-window</t>
+        </is>
+      </c>
+      <c r="E325" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-33/pygame-window.py</t>
+        </is>
+      </c>
+      <c r="F325" s="52" t="inlineStr">
+        <is>
+          <t>M6L1 Activity 1: Pygame Window</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B326" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C326" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 33 – Let's Begin with Pygame</t>
+        </is>
+      </c>
+      <c r="D326" s="52" t="inlineStr">
+        <is>
+          <t>add-image-to-the-screen</t>
+        </is>
+      </c>
+      <c r="E326" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-33/add-image-to-the-screen.py</t>
+        </is>
+      </c>
+      <c r="F326" s="52" t="inlineStr">
+        <is>
+          <t>M6L1 Activity 2: Add Image to the Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="54" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B327" s="54" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C327" s="54" t="inlineStr">
+        <is>
+          <t>Lesson 33 – Let's Begin with Pygame</t>
+        </is>
+      </c>
+      <c r="D327" s="54" t="inlineStr">
+        <is>
+          <t>my-first-game-screen</t>
+        </is>
+      </c>
+      <c r="E327" s="55" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/assignments/my-first-game-screen/my-first-game-screen.py</t>
+        </is>
+      </c>
+      <c r="F327" s="54" t="inlineStr">
+        <is>
+          <t>M6L1 ACP : My First Game Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B328" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C328" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Basic Game Building Concepts</t>
+        </is>
+      </c>
+      <c r="D328" s="52" t="inlineStr">
+        <is>
+          <t>draw-a-rectangle</t>
+        </is>
+      </c>
+      <c r="E328" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-34/draw-a-rectangle.py</t>
+        </is>
+      </c>
+      <c r="F328" s="52" t="inlineStr">
+        <is>
+          <t>M6L2 Activity 1: Draw a rectangle!</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B329" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C329" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Basic Game Building Concepts</t>
+        </is>
+      </c>
+      <c r="D329" s="52" t="inlineStr">
+        <is>
+          <t>hollow-and-solid-ball</t>
+        </is>
+      </c>
+      <c r="E329" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-34/hollow-and-solid-ball.py</t>
+        </is>
+      </c>
+      <c r="F329" s="52" t="inlineStr">
+        <is>
+          <t>M6L2 Activity 2: Hollow and Solid Ball</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B330" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C330" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Basic Game Building Concepts</t>
+        </is>
+      </c>
+      <c r="D330" s="52" t="inlineStr">
+        <is>
+          <t>color-changing-sprite</t>
+        </is>
+      </c>
+      <c r="E330" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-34/color-changing-sprite.py</t>
+        </is>
+      </c>
+      <c r="F330" s="52" t="inlineStr">
+        <is>
+          <t>M6L2 Activity 3: color changing sprite</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="54" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B331" s="54" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C331" s="54" t="inlineStr">
+        <is>
+          <t>Lesson 34 – Basic Game Building Concepts</t>
+        </is>
+      </c>
+      <c r="D331" s="54" t="inlineStr">
+        <is>
+          <t>add-elements-to-my-screen</t>
+        </is>
+      </c>
+      <c r="E331" s="55" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/assignments/add-elements-to-my-screen/add-elements-to-my-screen.py</t>
+        </is>
+      </c>
+      <c r="F331" s="54" t="inlineStr">
+        <is>
+          <t>M6L2 ACP : Add elements to my Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B332" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C332" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 35 – Let's Add Sprites</t>
+        </is>
+      </c>
+      <c r="D332" s="52" t="inlineStr">
+        <is>
+          <t>colorful-bounce</t>
+        </is>
+      </c>
+      <c r="E332" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-35/colorful-bounce.py</t>
+        </is>
+      </c>
+      <c r="F332" s="52" t="inlineStr">
+        <is>
+          <t>M6L3 Activity 1: Colorful bounce</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="54" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B333" s="54" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C333" s="54" t="inlineStr">
+        <is>
+          <t>Lesson 35 – Let's Add Sprites</t>
+        </is>
+      </c>
+      <c r="D333" s="54" t="inlineStr">
+        <is>
+          <t>add-sprites</t>
+        </is>
+      </c>
+      <c r="E333" s="55" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/assignments/add-sprites/add-sprites.py</t>
+        </is>
+      </c>
+      <c r="F333" s="54" t="inlineStr">
+        <is>
+          <t>M6L3 ACP : Add Sprites</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B334" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C334" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 36 – Let's Level Up The Game</t>
+        </is>
+      </c>
+      <c r="D334" s="52" t="inlineStr">
+        <is>
+          <t>sprite-collision</t>
+        </is>
+      </c>
+      <c r="E334" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-36/sprite-collision.py</t>
+        </is>
+      </c>
+      <c r="F334" s="52" t="inlineStr">
+        <is>
+          <t>M6L4 Activity 1: Sprite collision</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="54" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B335" s="54" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C335" s="54" t="inlineStr">
+        <is>
+          <t>Lesson 36 – Let's Level Up The Game</t>
+        </is>
+      </c>
+      <c r="D335" s="54" t="inlineStr">
+        <is>
+          <t>add-custom-event</t>
+        </is>
+      </c>
+      <c r="E335" s="55" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/assignments/add-custom-event/add-custom-event.py</t>
+        </is>
+      </c>
+      <c r="F335" s="54" t="inlineStr">
+        <is>
+          <t>M6L4 ACP: Add Custom Event</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B336" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C336" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 37 – Space Invader Project – Part 1</t>
+        </is>
+      </c>
+      <c r="D336" s="52" t="inlineStr">
+        <is>
+          <t>space-invader-game</t>
+        </is>
+      </c>
+      <c r="E336" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-37/space-invader-game.py</t>
+        </is>
+      </c>
+      <c r="F336" s="52" t="inlineStr">
+        <is>
+          <t>M6L5 Activity 1: Space Invader Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="54" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B337" s="54" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C337" s="54" t="inlineStr">
+        <is>
+          <t>Lesson 37 – Space Invader Project – Part 1</t>
+        </is>
+      </c>
+      <c r="D337" s="54" t="inlineStr">
+        <is>
+          <t>add-more-sprites</t>
+        </is>
+      </c>
+      <c r="E337" s="55" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/assignments/add-more-sprites/add-more-sprites.py</t>
+        </is>
+      </c>
+      <c r="F337" s="54" t="inlineStr">
+        <is>
+          <t>M6L5 ACP : Add more Sprites</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="52" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B338" s="52" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C338" s="52" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Space Invader Project – Part 2</t>
+        </is>
+      </c>
+      <c r="D338" s="52" t="inlineStr">
+        <is>
+          <t>space-invader-game</t>
+        </is>
+      </c>
+      <c r="E338" s="53" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/activities/lesson-38/space-invader-game.py</t>
+        </is>
+      </c>
+      <c r="F338" s="52" t="inlineStr">
+        <is>
+          <t>M6L6 Activity 1: Space Invader Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="54" t="inlineStr">
+        <is>
+          <t>PY-M6</t>
+        </is>
+      </c>
+      <c r="B339" s="54" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C339" s="54" t="inlineStr">
+        <is>
+          <t>Lesson 38 – Space Invader Project – Part 2</t>
+        </is>
+      </c>
+      <c r="D339" s="54" t="inlineStr">
+        <is>
+          <t>level-up-this-game</t>
+        </is>
+      </c>
+      <c r="E339" s="55" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m6/assignments/level-up-this-game/level-up-this-game.py</t>
+        </is>
+      </c>
+      <c r="F339" s="54" t="inlineStr">
+        <is>
+          <t>M6L6 ACP: Level Up this game</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10637,6 +11139,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E322" r:id="rId321"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E323" r:id="rId322"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E339" r:id="rId338"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Python M7 - GUI using Python Tkinter activities and ACPs
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="30">
+  <fills count="32">
     <fill>
       <patternFill/>
     </fill>
@@ -182,6 +182,16 @@
         <fgColor rgb="00F8BBD0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CE93D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF59D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -195,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -360,6 +370,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -727,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F339"/>
+  <dimension ref="A1:F355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10811,6 +10833,518 @@
       <c r="F339" s="54" t="inlineStr">
         <is>
           <t>M6L6 ACP: Level Up this game</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B340" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C340" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Widgets for Starters</t>
+        </is>
+      </c>
+      <c r="D340" s="56" t="inlineStr">
+        <is>
+          <t>pygame-window</t>
+        </is>
+      </c>
+      <c r="E340" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-39/pygame-window.py</t>
+        </is>
+      </c>
+      <c r="F340" s="56" t="inlineStr">
+        <is>
+          <t>M7L1 Activity 1: Pygame Window</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B341" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C341" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Widgets for Starters</t>
+        </is>
+      </c>
+      <c r="D341" s="56" t="inlineStr">
+        <is>
+          <t>getting-started-with-widgets</t>
+        </is>
+      </c>
+      <c r="E341" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-39/getting-started-with-widgets.py</t>
+        </is>
+      </c>
+      <c r="F341" s="56" t="inlineStr">
+        <is>
+          <t>M7L1 Activity 2: Getting started with widgets</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="58" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B342" s="58" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C342" s="58" t="inlineStr">
+        <is>
+          <t>Lesson 39 – Widgets for Starters</t>
+        </is>
+      </c>
+      <c r="D342" s="58" t="inlineStr">
+        <is>
+          <t>heres-the-product</t>
+        </is>
+      </c>
+      <c r="E342" s="59" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/assignments/heres-the-product/heres-the-product.py</t>
+        </is>
+      </c>
+      <c r="F342" s="58" t="inlineStr">
+        <is>
+          <t>M7L1 ACP : Here’s the product</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B343" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C343" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Tkinter Geometry Managers</t>
+        </is>
+      </c>
+      <c r="D343" s="56" t="inlineStr">
+        <is>
+          <t>number-pad</t>
+        </is>
+      </c>
+      <c r="E343" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-40/number-pad.py</t>
+        </is>
+      </c>
+      <c r="F343" s="56" t="inlineStr">
+        <is>
+          <t>M7L2 Activity 1: Number Pad</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B344" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C344" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Tkinter Geometry Managers</t>
+        </is>
+      </c>
+      <c r="D344" s="56" t="inlineStr">
+        <is>
+          <t>login-app</t>
+        </is>
+      </c>
+      <c r="E344" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-40/login-app.py</t>
+        </is>
+      </c>
+      <c r="F344" s="56" t="inlineStr">
+        <is>
+          <t>M7L2 Activity 2: Login App</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="58" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B345" s="58" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C345" s="58" t="inlineStr">
+        <is>
+          <t>Lesson 40 – Tkinter Geometry Managers</t>
+        </is>
+      </c>
+      <c r="D345" s="58" t="inlineStr">
+        <is>
+          <t>age-calculator-app</t>
+        </is>
+      </c>
+      <c r="E345" s="59" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/assignments/age-calculator-app/age-calculator-app.py</t>
+        </is>
+      </c>
+      <c r="F345" s="58" t="inlineStr">
+        <is>
+          <t>M7L2 ACP : Age Calculator App</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B346" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C346" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Where’s the event</t>
+        </is>
+      </c>
+      <c r="D346" s="56" t="inlineStr">
+        <is>
+          <t>event-handler</t>
+        </is>
+      </c>
+      <c r="E346" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-41/event-handler.py</t>
+        </is>
+      </c>
+      <c r="F346" s="56" t="inlineStr">
+        <is>
+          <t>M7L3 Activity 1: Event Handler</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B347" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C347" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Where’s the event</t>
+        </is>
+      </c>
+      <c r="D347" s="56" t="inlineStr">
+        <is>
+          <t>virus-detected</t>
+        </is>
+      </c>
+      <c r="E347" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-41/virus-detected.py</t>
+        </is>
+      </c>
+      <c r="F347" s="56" t="inlineStr">
+        <is>
+          <t>M7L3 Activity 2: Virus Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="58" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B348" s="58" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C348" s="58" t="inlineStr">
+        <is>
+          <t>Lesson 41 – Where’s the event</t>
+        </is>
+      </c>
+      <c r="D348" s="58" t="inlineStr">
+        <is>
+          <t>length-converter-app</t>
+        </is>
+      </c>
+      <c r="E348" s="59" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/assignments/length-converter-app/length-converter-app.py</t>
+        </is>
+      </c>
+      <c r="F348" s="58" t="inlineStr">
+        <is>
+          <t>M7L3 ACP : Length Converter App</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B349" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C349" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 42 – Let’s build a Text Editor</t>
+        </is>
+      </c>
+      <c r="D349" s="56" t="inlineStr">
+        <is>
+          <t>my-text-editor</t>
+        </is>
+      </c>
+      <c r="E349" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-42/my-text-editor.py</t>
+        </is>
+      </c>
+      <c r="F349" s="56" t="inlineStr">
+        <is>
+          <t>M7L4 Activity 1: My Text Editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="58" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B350" s="58" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C350" s="58" t="inlineStr">
+        <is>
+          <t>Lesson 42 – Let’s build a Text Editor</t>
+        </is>
+      </c>
+      <c r="D350" s="58" t="inlineStr">
+        <is>
+          <t>interest-calculator-app</t>
+        </is>
+      </c>
+      <c r="E350" s="59" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/assignments/interest-calculator-app/interest-calculator-app.py</t>
+        </is>
+      </c>
+      <c r="F350" s="58" t="inlineStr">
+        <is>
+          <t>M7L4 ACP: Interest Calculator App</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B351" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C351" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Denomination Calculator</t>
+        </is>
+      </c>
+      <c r="D351" s="56" t="inlineStr">
+        <is>
+          <t>lets-top-a-window</t>
+        </is>
+      </c>
+      <c r="E351" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-43/lets-top-a-window.py</t>
+        </is>
+      </c>
+      <c r="F351" s="56" t="inlineStr">
+        <is>
+          <t>M7L5 Activity 1: Let’s Top a Window</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B352" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C352" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Denomination Calculator</t>
+        </is>
+      </c>
+      <c r="D352" s="56" t="inlineStr">
+        <is>
+          <t>denomination-calculator</t>
+        </is>
+      </c>
+      <c r="E352" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-43/denomination-calculator.py</t>
+        </is>
+      </c>
+      <c r="F352" s="56" t="inlineStr">
+        <is>
+          <t>M7L5 Activity 2: Denomination Calculator</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="58" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B353" s="58" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C353" s="58" t="inlineStr">
+        <is>
+          <t>Lesson 43 – Denomination Calculator</t>
+        </is>
+      </c>
+      <c r="D353" s="58" t="inlineStr">
+        <is>
+          <t>password-strength-checker-app</t>
+        </is>
+      </c>
+      <c r="E353" s="59" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/assignments/password-strength-checker-app/password-strength-checker-app.py</t>
+        </is>
+      </c>
+      <c r="F353" s="58" t="inlineStr">
+        <is>
+          <t>M7L5 ACP : Password Strength Checker App</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="56" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B354" s="56" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C354" s="56" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Restaurant Management System</t>
+        </is>
+      </c>
+      <c r="D354" s="56" t="inlineStr">
+        <is>
+          <t>restaurant-management-system</t>
+        </is>
+      </c>
+      <c r="E354" s="57" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/activities/lesson-44/restaurant-management-system.py</t>
+        </is>
+      </c>
+      <c r="F354" s="56" t="inlineStr">
+        <is>
+          <t>M7L6 Activity 1: Restaurant Management System</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="58" t="inlineStr">
+        <is>
+          <t>PY-M7</t>
+        </is>
+      </c>
+      <c r="B355" s="58" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C355" s="58" t="inlineStr">
+        <is>
+          <t>Lesson 44 – Restaurant Management System</t>
+        </is>
+      </c>
+      <c r="D355" s="58" t="inlineStr">
+        <is>
+          <t>rock-paper-scissor-app</t>
+        </is>
+      </c>
+      <c r="E355" s="59" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m7/assignments/rock-paper-scissor-app/rock-paper-scissor-app.py</t>
+        </is>
+      </c>
+      <c r="F355" s="58" t="inlineStr">
+        <is>
+          <t>M7L6 ACP: Rock Paper Scissor App</t>
         </is>
       </c>
     </row>
@@ -11154,6 +11688,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E337" r:id="rId336"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E338" r:id="rId337"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E355" r:id="rId354"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Python M12 SQL activities, ACPs and projects
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="32">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
@@ -192,6 +192,21 @@
         <fgColor rgb="00FFF59D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0081D4FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCC80"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A5D6A7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -205,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -382,6 +397,24 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -749,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F355"/>
+  <dimension ref="A1:F372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11347,6 +11380,542 @@
           <t>M7L6 ACP: Rock Paper Scissor App</t>
         </is>
       </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B356" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C356" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 67 – SQL- CREATE TABLE</t>
+        </is>
+      </c>
+      <c r="D356" s="60" t="inlineStr">
+        <is>
+          <t>supplier-table</t>
+        </is>
+      </c>
+      <c r="E356" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-67/supplier-table.py</t>
+        </is>
+      </c>
+      <c r="F356" s="60" t="inlineStr">
+        <is>
+          <t>SQL1</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B357" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C357" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 67 – SQL- CREATE TABLE</t>
+        </is>
+      </c>
+      <c r="D357" s="60" t="inlineStr">
+        <is>
+          <t>salesman-and-orders-table</t>
+        </is>
+      </c>
+      <c r="E357" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-67/salesman-and-orders-table.py</t>
+        </is>
+      </c>
+      <c r="F357" s="60" t="inlineStr">
+        <is>
+          <t>SQL2</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B358" s="62" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C358" s="62" t="inlineStr">
+        <is>
+          <t>Lesson 67 – SQL- CREATE TABLE</t>
+        </is>
+      </c>
+      <c r="D358" s="62" t="inlineStr">
+        <is>
+          <t>create-table</t>
+        </is>
+      </c>
+      <c r="E358" s="63" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/create-table/create-table.py</t>
+        </is>
+      </c>
+      <c r="F358" s="62" t="inlineStr">
+        <is>
+          <t>Create Table</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B359" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C359" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 68 – SQL-OPERATORS</t>
+        </is>
+      </c>
+      <c r="D359" s="60" t="inlineStr">
+        <is>
+          <t>student-table-queries</t>
+        </is>
+      </c>
+      <c r="E359" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-68/student-table-queries.py</t>
+        </is>
+      </c>
+      <c r="F359" s="60" t="inlineStr">
+        <is>
+          <t>SQL 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B360" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C360" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 68 – SQL-OPERATORS</t>
+        </is>
+      </c>
+      <c r="D360" s="60" t="inlineStr">
+        <is>
+          <t>product-price-queries</t>
+        </is>
+      </c>
+      <c r="E360" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-68/product-price-queries.py</t>
+        </is>
+      </c>
+      <c r="F360" s="60" t="inlineStr">
+        <is>
+          <t>SQL 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B361" s="62" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C361" s="62" t="inlineStr">
+        <is>
+          <t>Lesson 68 – SQL-OPERATORS</t>
+        </is>
+      </c>
+      <c r="D361" s="62" t="inlineStr">
+        <is>
+          <t>operators</t>
+        </is>
+      </c>
+      <c r="E361" s="63" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/operators/operators.py</t>
+        </is>
+      </c>
+      <c r="F361" s="62" t="inlineStr">
+        <is>
+          <t>Operators</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B362" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C362" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 69 – SQL- AGGREGATE FUNCTIONS</t>
+        </is>
+      </c>
+      <c r="D362" s="60" t="inlineStr">
+        <is>
+          <t>product-table-and-aggregate-queries</t>
+        </is>
+      </c>
+      <c r="E362" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-69/product-table-and-aggregate-queries.py</t>
+        </is>
+      </c>
+      <c r="F362" s="60" t="inlineStr">
+        <is>
+          <t>SQL5</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B363" s="62" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C363" s="62" t="inlineStr">
+        <is>
+          <t>Lesson 69 – SQL- AGGREGATE FUNCTIONS</t>
+        </is>
+      </c>
+      <c r="D363" s="62" t="inlineStr">
+        <is>
+          <t>aggregate-functions</t>
+        </is>
+      </c>
+      <c r="E363" s="63" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/aggregate-functions/aggregate-functions.py</t>
+        </is>
+      </c>
+      <c r="F363" s="62" t="inlineStr">
+        <is>
+          <t>Aggregate Functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B364" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C364" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
+        </is>
+      </c>
+      <c r="D364" s="60" t="inlineStr">
+        <is>
+          <t>nobel-prize-winners-table-and-queries</t>
+        </is>
+      </c>
+      <c r="E364" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-70/nobel-prize-winners-table-and-queries.py</t>
+        </is>
+      </c>
+      <c r="F364" s="60" t="inlineStr">
+        <is>
+          <t>SQL6</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B365" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C365" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
+        </is>
+      </c>
+      <c r="D365" s="60" t="inlineStr">
+        <is>
+          <t>department-table-and-aggregate-queries</t>
+        </is>
+      </c>
+      <c r="E365" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-70/department-table-and-aggregate-queries.py</t>
+        </is>
+      </c>
+      <c r="F365" s="60" t="inlineStr">
+        <is>
+          <t>SQL6</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B366" s="62" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C366" s="62" t="inlineStr">
+        <is>
+          <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
+        </is>
+      </c>
+      <c r="D366" s="62" t="inlineStr">
+        <is>
+          <t>sort-and-filter</t>
+        </is>
+      </c>
+      <c r="E366" s="63" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/sort-and-filter/sort-and-filter.py</t>
+        </is>
+      </c>
+      <c r="F366" s="62" t="inlineStr">
+        <is>
+          <t>Sortt &amp; Filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B367" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C367" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 71 – SQL Capstone Project-1</t>
+        </is>
+      </c>
+      <c r="D367" s="60" t="inlineStr">
+        <is>
+          <t>sql-capstone-project-1</t>
+        </is>
+      </c>
+      <c r="E367" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-71/sql-capstone-project-1.py</t>
+        </is>
+      </c>
+      <c r="F367" s="60" t="inlineStr">
+        <is>
+          <t>capstone project</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B368" s="62" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C368" s="62" t="inlineStr">
+        <is>
+          <t>Lesson 71 – SQL Capstone Project-1</t>
+        </is>
+      </c>
+      <c r="D368" s="62" t="inlineStr">
+        <is>
+          <t>capstone-project-1</t>
+        </is>
+      </c>
+      <c r="E368" s="63" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/capstone-project-1/capstone-project-1.py</t>
+        </is>
+      </c>
+      <c r="F368" s="62" t="inlineStr">
+        <is>
+          <t>Capstone Project 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="60" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B369" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C369" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 72 – SQL Capstone Project -2</t>
+        </is>
+      </c>
+      <c r="D369" s="60" t="inlineStr">
+        <is>
+          <t>new-york-restaurant</t>
+        </is>
+      </c>
+      <c r="E369" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-72/new-york-restaurant.py</t>
+        </is>
+      </c>
+      <c r="F369" s="60" t="inlineStr">
+        <is>
+          <t>New York Restaurant</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B370" s="62" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C370" s="62" t="inlineStr">
+        <is>
+          <t>Lesson 72 – SQL Capstone Project -2</t>
+        </is>
+      </c>
+      <c r="D370" s="62" t="inlineStr">
+        <is>
+          <t>capstone-project-2</t>
+        </is>
+      </c>
+      <c r="E370" s="63" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/capstone-project-2/capstone-project-2.py</t>
+        </is>
+      </c>
+      <c r="F370" s="62" t="inlineStr">
+        <is>
+          <t>Capstone Project 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="64" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B371" s="64" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C371" s="64" t="inlineStr">
+        <is>
+          <t>Lesson 69 – SQL- AGGREGATE FUNCTIONS</t>
+        </is>
+      </c>
+      <c r="D371" s="64" t="inlineStr">
+        <is>
+          <t>zoo-explorer</t>
+        </is>
+      </c>
+      <c r="E371" s="65" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/projects/lesson-69/zoo-explorer.py</t>
+        </is>
+      </c>
+      <c r="F371" s="64" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="64" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B372" s="64" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C372" s="64" t="inlineStr">
+        <is>
+          <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
+        </is>
+      </c>
+      <c r="D372" s="64" t="inlineStr">
+        <is>
+          <t>book-club-explorer</t>
+        </is>
+      </c>
+      <c r="E372" s="65" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/projects/lesson-70/book-club-explorer.py</t>
+        </is>
+      </c>
+      <c r="F372" s="64" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11704,6 +12273,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E353" r:id="rId352"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E354" r:id="rId353"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E372" r:id="rId371"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Move book-club-explorer into lesson-70 activities and map it to the SQL6 SQL 7 form field
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -11702,192 +11702,196 @@
       </c>
     </row>
     <row r="366">
-      <c r="A366" s="62" t="inlineStr">
+      <c r="A366" s="60" t="inlineStr">
         <is>
           <t>PY-M12</t>
         </is>
       </c>
-      <c r="B366" s="62" t="inlineStr">
+      <c r="B366" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C366" s="60" t="inlineStr">
+        <is>
+          <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
+        </is>
+      </c>
+      <c r="D366" s="60" t="inlineStr">
+        <is>
+          <t>book-club-explorer</t>
+        </is>
+      </c>
+      <c r="E366" s="61" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-70/book-club-explorer.py</t>
+        </is>
+      </c>
+      <c r="F366" s="60" t="inlineStr">
+        <is>
+          <t>SQL6	SQL 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="62" t="inlineStr">
+        <is>
+          <t>PY-M12</t>
+        </is>
+      </c>
+      <c r="B367" s="62" t="inlineStr">
         <is>
           <t>ACP</t>
         </is>
       </c>
-      <c r="C366" s="62" t="inlineStr">
+      <c r="C367" s="62" t="inlineStr">
         <is>
           <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
         </is>
       </c>
-      <c r="D366" s="62" t="inlineStr">
+      <c r="D367" s="62" t="inlineStr">
         <is>
           <t>sort-and-filter</t>
         </is>
       </c>
-      <c r="E366" s="63" t="inlineStr">
+      <c r="E367" s="63" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/sort-and-filter/sort-and-filter.py</t>
         </is>
       </c>
-      <c r="F366" s="62" t="inlineStr">
+      <c r="F367" s="62" t="inlineStr">
         <is>
           <t>Sortt &amp; Filter</t>
         </is>
       </c>
     </row>
-    <row r="367">
-      <c r="A367" s="60" t="inlineStr">
+    <row r="368">
+      <c r="A368" s="60" t="inlineStr">
         <is>
           <t>PY-M12</t>
         </is>
       </c>
-      <c r="B367" s="60" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C367" s="60" t="inlineStr">
+      <c r="B368" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C368" s="60" t="inlineStr">
         <is>
           <t>Lesson 71 – SQL Capstone Project-1</t>
         </is>
       </c>
-      <c r="D367" s="60" t="inlineStr">
+      <c r="D368" s="60" t="inlineStr">
         <is>
           <t>sql-capstone-project-1</t>
         </is>
       </c>
-      <c r="E367" s="61" t="inlineStr">
+      <c r="E368" s="61" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-71/sql-capstone-project-1.py</t>
         </is>
       </c>
-      <c r="F367" s="60" t="inlineStr">
+      <c r="F368" s="60" t="inlineStr">
         <is>
           <t>capstone project</t>
         </is>
       </c>
     </row>
-    <row r="368">
-      <c r="A368" s="62" t="inlineStr">
+    <row r="369">
+      <c r="A369" s="62" t="inlineStr">
         <is>
           <t>PY-M12</t>
         </is>
       </c>
-      <c r="B368" s="62" t="inlineStr">
+      <c r="B369" s="62" t="inlineStr">
         <is>
           <t>ACP</t>
         </is>
       </c>
-      <c r="C368" s="62" t="inlineStr">
+      <c r="C369" s="62" t="inlineStr">
         <is>
           <t>Lesson 71 – SQL Capstone Project-1</t>
         </is>
       </c>
-      <c r="D368" s="62" t="inlineStr">
+      <c r="D369" s="62" t="inlineStr">
         <is>
           <t>capstone-project-1</t>
         </is>
       </c>
-      <c r="E368" s="63" t="inlineStr">
+      <c r="E369" s="63" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/capstone-project-1/capstone-project-1.py</t>
         </is>
       </c>
-      <c r="F368" s="62" t="inlineStr">
+      <c r="F369" s="62" t="inlineStr">
         <is>
           <t>Capstone Project 1</t>
         </is>
       </c>
     </row>
-    <row r="369">
-      <c r="A369" s="60" t="inlineStr">
+    <row r="370">
+      <c r="A370" s="60" t="inlineStr">
         <is>
           <t>PY-M12</t>
         </is>
       </c>
-      <c r="B369" s="60" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C369" s="60" t="inlineStr">
+      <c r="B370" s="60" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C370" s="60" t="inlineStr">
         <is>
           <t>Lesson 72 – SQL Capstone Project -2</t>
         </is>
       </c>
-      <c r="D369" s="60" t="inlineStr">
+      <c r="D370" s="60" t="inlineStr">
         <is>
           <t>new-york-restaurant</t>
         </is>
       </c>
-      <c r="E369" s="61" t="inlineStr">
+      <c r="E370" s="61" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/activities/lesson-72/new-york-restaurant.py</t>
         </is>
       </c>
-      <c r="F369" s="60" t="inlineStr">
+      <c r="F370" s="60" t="inlineStr">
         <is>
           <t>New York Restaurant</t>
         </is>
       </c>
     </row>
-    <row r="370">
-      <c r="A370" s="62" t="inlineStr">
+    <row r="371">
+      <c r="A371" s="62" t="inlineStr">
         <is>
           <t>PY-M12</t>
         </is>
       </c>
-      <c r="B370" s="62" t="inlineStr">
+      <c r="B371" s="62" t="inlineStr">
         <is>
           <t>ACP</t>
         </is>
       </c>
-      <c r="C370" s="62" t="inlineStr">
+      <c r="C371" s="62" t="inlineStr">
         <is>
           <t>Lesson 72 – SQL Capstone Project -2</t>
         </is>
       </c>
-      <c r="D370" s="62" t="inlineStr">
+      <c r="D371" s="62" t="inlineStr">
         <is>
           <t>capstone-project-2</t>
         </is>
       </c>
-      <c r="E370" s="63" t="inlineStr">
+      <c r="E371" s="63" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/assignments/capstone-project-2/capstone-project-2.py</t>
         </is>
       </c>
-      <c r="F370" s="62" t="inlineStr">
+      <c r="F371" s="62" t="inlineStr">
         <is>
           <t>Capstone Project 2</t>
         </is>
       </c>
-    </row>
-    <row r="371">
-      <c r="A371" s="64" t="inlineStr">
-        <is>
-          <t>PY-M12</t>
-        </is>
-      </c>
-      <c r="B371" s="64" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="C371" s="64" t="inlineStr">
-        <is>
-          <t>Lesson 69 – SQL- AGGREGATE FUNCTIONS</t>
-        </is>
-      </c>
-      <c r="D371" s="64" t="inlineStr">
-        <is>
-          <t>zoo-explorer</t>
-        </is>
-      </c>
-      <c r="E371" s="65" t="inlineStr">
-        <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/projects/lesson-69/zoo-explorer.py</t>
-        </is>
-      </c>
-      <c r="F371" s="64" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" s="64" t="inlineStr">
@@ -11902,17 +11906,17 @@
       </c>
       <c r="C372" s="64" t="inlineStr">
         <is>
-          <t>Lesson 70 – SQL- GROUPING,FILTERING &amp; SORTING</t>
+          <t>Lesson 69 – SQL- AGGREGATE FUNCTIONS</t>
         </is>
       </c>
       <c r="D372" s="64" t="inlineStr">
         <is>
-          <t>book-club-explorer</t>
+          <t>zoo-explorer</t>
         </is>
       </c>
       <c r="E372" s="65" t="inlineStr">
         <is>
-          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/projects/lesson-70/book-club-explorer.py</t>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/python_m12/projects/lesson-69/zoo-explorer.py</t>
         </is>
       </c>
       <c r="F372" s="64" t="inlineStr"/>

</xml_diff>